<commit_message>
Enhance Jupyter notebook with evaluation criteria and product processing updates
- Introduced quality and objective criteria for product evaluation.
- Updated execution counts for code cells to maintain proper order.
- Expanded product processing output to include all 50 items.
- Adjusted generated description statistics for accuracy in results.
- Modified product description content for improved clarity.
</commit_message>
<xml_diff>
--- a/assignment_01.xlsx
+++ b/assignment_01.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,17 +521,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unlock limitless possibilities with the Apple iPhone 15 Pro. Powered by the lightning-fast A17 Pro chip, this marvel of engineering delivers seamless performance and lightning-fast speeds. Enjoy vibrant visuals on the stunning 120 Hz ProMotion display, complemented by the durability of titanium and Ceramic Shield glass. Rapidly recharge your battery with USB-C fast charging. This sleek and compact powerhouse is also backed by a 1-year limited warranty, giving you peace of mind and the freedom to explore your creativity. Elevate your mobile experience with the iPhone 15 Pro.</t>
+          <t>"Upgrade your mobile experience with the Apple iPhone 15 Pro. Powered by the A17 Pro chip, this device delivers lightning-fast performance and seamless multitasking. The stunning 120 Hz ProMotion display brings immersive graphics and effortless scrolling. Plus, fast USB-C charging means you can power up quickly. Crafted with durable titanium and shatter-resistant Ceramic Shield glass, the iPhone 15 Pro is a sleek and durable companion for on-the-go adventurous types. Backed by a comprehensive 1-year warranty, you can buy with confidence."</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>5587</v>
+        <v>11975</v>
       </c>
       <c r="G2" t="n">
         <v>200</v>
       </c>
       <c r="H2" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -565,17 +565,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Elevate your mobile experience with the Samsung Galaxy S24 Ultra. Capture life's moments in breathtaking detail with its 200 MP camera, perfect for enthusiasts and professionals alike. The S-Pen stylus brings limitless creativity to your fingertips, and the vibrant 120 Hz AMOLED display ensures seamless visuals. Sustainably sourced and crafted with a strong Armor Aluminum frame and durable Gorilla Glass Victus, this device is both built to last and kind to the planet. Confidently own the latest technology with a 1-year limited warranty.</t>
+          <t>"Unlock your creativity with the Samsung Galaxy S24 Ultra, the ultimate smartphone for content creators and tech enthusiasts alike. This powerhouse boasts a 200 MP camera for breathtakingly clear photos and videos, paired with S-Pen support for a more expressive artistic experience. Its stunning 120 Hz AMOLED display provides a seamless visual treat. Crafted with eco-conscious materials, including sustainably sourced Armor Aluminum and Gorilla Glass Victus, this device is as functional as it is responsible. Enjoy a 1-year limited warranty and discover new heights of innovation."</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4877</v>
+        <v>9583</v>
       </c>
       <c r="G3" t="n">
         <v>203</v>
       </c>
       <c r="H3" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -586,6 +586,2118 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Google Pixel 8 Pro</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>features: Tensor G3 chip, Magic Eraser, 50 MP camera; rating: 4.7/5</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>matte glass back, aluminum frame</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>"Unlock the power of unparalleled photography with the Google Pixel 8 Pro. Equipped with the innovative Tensor G3 chip, this smartphone delivers stunning images with its 50 MP camera. The Magic Eraser feature takes removing unwanted objects to the next level. Durable and sleek, the matte glass back and aluminum frame ensure a comfortable grip. With a rating of 4.7/5, users rave about this device. Experience seamless performance, effortlessly capture life's moments, and enjoy peace of mind with the 1-year limited warranty."</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>14984</v>
+      </c>
+      <c r="G4" t="n">
+        <v>202</v>
+      </c>
+      <c r="H4" t="n">
+        <v>109</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sony WH-1000XM5 Headphones</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>features: active noise cancelling, 30 hr battery, Bluetooth 5.2; capacity: large</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>synthetic leather earcups</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Escape the noise with the Sony WH-1000XM5 Headphones. These revolutionary headphones boast exceptional active noise-cancelling technology, effortlessly silencing distractions. With a whopping 30-hour battery life, you can enjoy uninterrupted listening on long flights or busy commutes. pairs seamlessly via Bluetooth 5.2. The large capacity storage means you can store your music, podcasts, and audiobooks with plenty of room for all your favourites. Upgrade your listening experience with the Sony WH-1000XM5 - order now and discover a world of crisp, clear sound.</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>9036</v>
+      </c>
+      <c r="G5" t="n">
+        <v>201</v>
+      </c>
+      <c r="H5" t="n">
+        <v>116</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bose QuietComfort Ultra Earbuds</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>features: CustomTune sound calibration, ANC, IPX4; award-winning design</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>silicone ear tips</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Immerse yourself in the perfect blend of sound and silence with the Bose QuietComfort Ultra Earbuds. Our state-of-the-art earbuds use CustomTune sound calibration to deliver a personalized audio experience that's tailored to your unique hearing. With Advanced Noise Cancellation (ANC) and IPX4 water and sweat resistance, you can enjoy your favorite tunes in any setting. Durable silicone ear tips fit comfortably in your ear, and a 1-year limited warranty gives you peace of mind. Elevate your listening experience with QuietComfort Ultra Earbuds.</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>7361</v>
+      </c>
+      <c r="G6" t="n">
+        <v>194</v>
+      </c>
+      <c r="H6" t="n">
+        <v>115</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Amazon Echo Dot (5th Gen)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>features: Alexa voice assistant, temperature sensor, improved bass; sustainably sourced</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>recycled fabric mesh</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>"Get ready to transform your home with the Amazon Echo Dot (5th Gen). This compact powerhouse features Alexa, the world's most intelligent voice assistant, at its core. With a built-in temperature sensor, you'll stay cozy and connected, while improved bass ensures you'll always get the beat. Sustainably sourced from recycled materials, this eco-friendly smart speaker also boasts a stylish fabric mesh design. Plus, enjoy peace of mind with a 1-year limited warranty. Upgrade your space and elevate your life with this cutting-edge innovation."</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>6481</v>
+      </c>
+      <c r="G7" t="n">
+        <v>192</v>
+      </c>
+      <c r="H7" t="n">
+        <v>109</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dell XPS 13 9310 Laptop</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>features: 13.4″ FHD+ display, Intel Core i5, Thunderbolt 4; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CNC aluminum &amp; carbon-fiber palmrest</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1-year limited hardware warranty</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Elevate your productivity on-the-go with the Dell XPS 13 9310 Laptop. This compact powerhouse features a stunning 13.4" FHD+ display, plus a responsive Intel Core i5 processor and fast Thunderbolt 4 connectivity. Crafted with premium materials, including durable CNC aluminum and a carbon-fiber palmrest, this sleek laptop is built to withstand the rigors of travel. Enjoy worry-free computing with a 1-year limited hardware warranty – get ready to take your work to the next level, anywhere, anytime.</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>6205</v>
+      </c>
+      <c r="G8" t="n">
+        <v>210</v>
+      </c>
+      <c r="H8" t="n">
+        <v>112</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Apple MacBook Air 13″ (M3)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>features: M3 chip, 18-hour battery, 1080p camera; energy efficient</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>recycled aluminum unibody</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Create and unleash your creativity on the go with the Apple MacBook Air 13″ (M3). Powered by the efficient M3 chip, this stunning laptop delivers all-day performance, up to 18 hours of battery life, and a vibrant 1080p camera perfect for video conferencing. Made from 100% recycled aluminum, you can feel good about your purchase while staying productive, wherever inspiration strikes. Plus, enjoy peace of mind with a 1-year limited warranty.</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>6735</v>
+      </c>
+      <c r="G9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H9" t="n">
+        <v>97</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Microsoft Surface Pro 10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>features: Intel Core Ultra, detachable keyboard, 13″ PixelSense; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>magnesium alloy chassis</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Take your productivity on-the-go to the next level with the Microsoft Surface Pro 10! This ultra-compact powerhouse features a stunning 13-inch PixelSense display and a lightning-fast Intel Core Ultra processor. Plus, detach the keyboard and get creative - sketch, write, or browse with ease. Crafted with a durable magnesium alloy chassis, this versatile tablet is built to last. With a 1-year limited warranty, you can trust that your Surface Pro 10 has got your back. Work on any surface, anywhere.</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>8158</v>
+      </c>
+      <c r="G10" t="n">
+        <v>194</v>
+      </c>
+      <c r="H10" t="n">
+        <v>106</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Garmin Forerunner 255</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>features: multi-band GPS, HRV status, 14-day battery; rating: 4.7/5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>fiber-reinforced polymer</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Take your training to the next level with the Garmin Forerunner 255, a cutting-edge GPS watch that tracks your every move. Savings on each intense workout, monitor your heart rate variation (HRV) status to optimize recovery, and push your limits with up to 14 days of battery life. This rugged timepiece features a lightweight, fiber-reinforced design and a 1-year limited warranty. Upgrade your fitness routine with unrivaled accuracy and discover a performance boost you never knew you needed.</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>6520</v>
+      </c>
+      <c r="G11" t="n">
+        <v>201</v>
+      </c>
+      <c r="H11" t="n">
+        <v>103</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fitbit Charge 6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>features: heart-rate monitor, built-in GPS, 7-day battery; color options: multiple</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>aluminum case</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>"Take control of your fitness journey with the Fitbit Charge 6! This sleek and durable device tracks your progress with a built-in GPS and continuous heart-rate monitoring. Enjoy up to 7 days of battery life, so you can track your fitness goals without worrying about keeping it charged. Available in a variety of colors to suit your style, the Fitbit Charge 6 comes with a 1-year limited warranty for peace of mind. Get fit, feel focused, and stick to your goals with this reliable and feature-packed fitness tracker."</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>12951</v>
+      </c>
+      <c r="G12" t="n">
+        <v>193</v>
+      </c>
+      <c r="H12" t="n">
+        <v>109</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GoPro HERO12 Black</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>features: 5.3K60 video, HyperSmooth 6.0, waterproof 10 m; capacity: large</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rugged polycarbonate</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Capture life's most epic moments with confidence! The GoPro HERO12 Black is the ultimate action camera, delivering stunning 5.3K60 video and silky-smooth footage with HyperSmooth 6.0. Don't worry about the elements - it's waterproof up to 10m, and its rugged polycarbonate body can withstand rough handling. Dive in, ski down, or hike up - with a 1-year limited warranty, you can focus on the adventure, not worrying about your gear.</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>7715</v>
+      </c>
+      <c r="G13" t="n">
+        <v>201</v>
+      </c>
+      <c r="H13" t="n">
+        <v>103</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DJI Mini 4 Pro Drone</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>features: 4K/60fps, omnidirectional obstacle sensing, &lt;250 g; rating: 4.7/5</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>composite plastic</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Take to the skies with the ultra-light DJI Mini 4 Pro Drone! Weighing under 250g, this portable powerhouse captures stunning 4K/60fps footage and features omnidirectional obstacle sensing for safe flight. With a 4.7/5 rating, you can trust it to deliver exceptional results. Durable composite plastic construction ensures long-lasting use. Backed by a 1-year limited warranty, make sure to capture every precious moment with this top-notch drone. Perfect for creators and travelers alike, get ready to soar to new heights!</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>11969</v>
+      </c>
+      <c r="G14" t="n">
+        <v>203</v>
+      </c>
+      <c r="H14" t="n">
+        <v>115</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Nintendo Switch OLED</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>features: 7″ OLED screen, docked &amp; handheld modes, 64 GB storage; capacity: large</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>plastic chassis</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Take your gaming to the next level with the Nintendo Switch OLED. This powerhouse features a vibrant 7" OLED screen, perfect for immersive gameplay. Explore new worlds in docked mode, or take the fun on the go with handheld mode. Boot up to 64GB of storage, plenty of room for your favourite games and memories. Plus, a durable plastic chassis keeps your console looking great. Enjoy a year of worry-free gaming with our limited one-year warranty. Get ready to level up your gaming experience!</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>7965</v>
+      </c>
+      <c r="G15" t="n">
+        <v>194</v>
+      </c>
+      <c r="H15" t="n">
+        <v>103</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PlayStation 5 Slim</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>features: ray tracing, haptic feedback controller, 1 TB SSD; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>plastic shell</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Play a new level of immersive gaming with the PlayStation 5 Slim. Experience stunning visuals with ray tracing, feel every vibration with our haptic feedback controller, and load games lightning-fast with the 1 TB SSD. Plus, enjoy hours of uninterrupted gaming with our long-lasting battery. At 30% lighter, our slim design fits perfectly in any entertainment space. With a 1-year limited warranty, you can shop with confidence. Revolutionize your gaming experience with the PlayStation 5 Slim today!</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>9493</v>
+      </c>
+      <c r="G16" t="n">
+        <v>192</v>
+      </c>
+      <c r="H16" t="n">
+        <v>100</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Xbox Series X</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>features: 12 TFLOPS GPU, 1 TB SSD, 4K @ 120 Hz; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>matte black casing</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Elevate your gaming experience with the Xbox Series X. This powerhouse console boasts a 12 TFLOPS GPU, delivering stunning 4K graphics at 120 Hz, while its 1 TB SSD ensures seamless gameplay and near-instant load times. The durable matte black casing is designed to withstand the rigors of frequent play. Plus, enjoy long-lasting battery life and worry about resources, thanks to Microsoft's 1-year limited warranty, giving you peace of mind and freedom to focus on enjoying the latest titles.</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>7601</v>
+      </c>
+      <c r="G17" t="n">
+        <v>199</v>
+      </c>
+      <c r="H17" t="n">
+        <v>105</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Instant Pot Duo 6-Quart</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>features: 7-in-1 multicooker, stainless steel inner pot, 1000 W heating; weight: light</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>18/8 stainless steel</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Cook smarter, not harder, with the Instant Pot Duo 6-Quart! This 7-in-1 multicooker is a kitchen game-changer, allowing you to pressure cook, slow cook, sauté, steam, yam, and even make yogurt. The stainless steel inner pot is durable and dishwasher safe, while the 1000 W heating ensures fast cooking times. Plus, at just a few pounds, it's easy to lift and store. Backed by a 1-year limited warranty, you can trust your new Instant Pot Duo will become a trusted companion in the kitchen.</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>9455</v>
+      </c>
+      <c r="G18" t="n">
+        <v>206</v>
+      </c>
+      <c r="H18" t="n">
+        <v>123</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Keurig K-Supreme Plus Smart</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>features: multistream extraction, BrewID, 78 oz reservoir; capacity: large</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>brushed stainless steel accents</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Elevate your coffee experience with the Keurig K-Supreme Plus Smart! This sleek brewer boasts a massive 78 oz reservoir and multistream extraction, delivering rich and full-bodied flavors with ease. With BrewID technology, you'll get perfect results every time. Plus, the brushed stainless steel accents add a touch of modern style to your kitchen. Get 1 year of peace of mind with our limited warranty. Upgrade your daily coffee routine with the K-Supreme Plus Smart – order yours today!</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>6638</v>
+      </c>
+      <c r="G19" t="n">
+        <v>197</v>
+      </c>
+      <c r="H19" t="n">
+        <v>105</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Vitamix 5200 Blender</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>features: variable speed, 2-hp motor, self-cleaning; sustainably sourced</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BPA-free Tritan jar</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>7-year warranty</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Unlock the power of nutrient-rich blending with the Vitamix 5200 Blender. This heavy-duty machine features a robust 2-hp motor and variable speed control, tackling everything from frozen sorbet to hot soups. The BPA-free Tritan jar withstands rigorous use, and the self-cleaning design makes maintenance a breeze. Enjoy peace of mind with our 7-year warranty. Join the blending revolution and experience unparalleled performance, sustainably sourced for a healthier you.</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>5576</v>
+      </c>
+      <c r="G20" t="n">
+        <v>197</v>
+      </c>
+      <c r="H20" t="n">
+        <v>97</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Dyson V15 Detect Vacuum</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>features: laser dust detection, HEPA filtration, 60-min run-time; energy efficient</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>polycarbonate &amp; aluminum</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2-year parts &amp; labor</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>"Say goodbye to dusty messes with the Dyson V15 Detect Vacuum! This sleek and powerful tool utilizes laser dust detection to pinpoint hidden dirt and debris, while its HEPA filtration system captures 99.97% of microscopic particles. Enjoy up to 60 minutes of continuous cleaning and rest assured with a 2-year parts and labor warranty. Plus, its energy-efficient design keeps your wallet happy and the planet grateful. Boost your cleaning routine with the innovative Dyson V15 Detect Vacuum!"</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>5930</v>
+      </c>
+      <c r="G21" t="n">
+        <v>197</v>
+      </c>
+      <c r="H21" t="n">
+        <v>100</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>iRobot Roomba j7+</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>features: PrecisionVision navigation, self-emptying Clean Base, Alexa; award-winning design</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>plastic housing</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Meet the future of cleaning with the iRobot Roomba j7+! This sleek, award-winning robot vacuum navigates with ease thanks to PrecisionVision, ensuring a spotless floor. When it's done, simply let it empty itself into the Clean Base – no more dusty bin cleaning! Plus, control it with ease via Alexa. Backed by a 1-year limited warranty, the Roomba j7+ is the ultimate low-maintenance solution for a cleaner, happier home.</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>5582</v>
+      </c>
+      <c r="G22" t="n">
+        <v>192</v>
+      </c>
+      <c r="H22" t="n">
+        <v>98</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Yeti Rambler 20 oz Tumbler</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>features: double-wall vacuum insulated, MagSlider lid; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>kitchen-grade stainless steel</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>5-year warranty</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Take your daily grind to the next level with the Yeti Rambler 20 oz Tumbler. This compact workhorse is built to last, thanks to kitchen-grade stainless steel and a 5-year warranty. The double-wall vacuum insulation keeps drinks hot for hours, while the MagSlider lid seals in the goodness and prevents spills. Whether you're sipping coffee or tea on-the-go, this rambler is designed to keep up with your active lifestyle. Upgrade your hydration routine today!</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>5739</v>
+      </c>
+      <c r="G23" t="n">
+        <v>195</v>
+      </c>
+      <c r="H23" t="n">
+        <v>101</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Stanley Quencher H2.0 40 oz</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>features: vacuum insulated, flow-state lid, cup-holder friendly; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>recycled stainless steel</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Stay hydrated on-the-go with the Stanley Quencher H2.0 40oz! This incredible cup is built to keep up with your active lifestyle. The vacuum insulated design and flow-state lid allow for easy sipping and secure closures, while the cup-holder friendly design fits seamlessly into your vehicle or desk. Made from lightweight, recycled stainless steel, this durable bottle withstands even the toughest adventures. Plus, with a lifetime warranty, you can trust it'll be your go-to hydration companion for years to come.</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>6149</v>
+      </c>
+      <c r="G24" t="n">
+        <v>195</v>
+      </c>
+      <c r="H24" t="n">
+        <v>105</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hydro Flask 32 oz Wide Mouth</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>features: TempShield insulation, Color Last powder coat; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>pro-grade stainless steel</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>"Keep your drinks hot or cold for hours with the Hydro Flask 32 oz Wide Mouth! Made from pro-grade stainless steel, this BPA-free bottle is built to last with a compact design that fits perfectly in your hand or car cup holder. The TempShield insulation keeps your drinks at the perfect temperature, while the Color Last powder coat makes it shine. And don't worry - with our lifetime warranty, you can enjoy your Hydro Flask worry-free!"</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>5515</v>
+      </c>
+      <c r="G25" t="n">
+        <v>189</v>
+      </c>
+      <c r="H25" t="n">
+        <v>92</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Contigo Autoseal West Loop 16 oz</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>features: autoseal spill-proof lid, double-wall insulation; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>stainless steel</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Stay hydrated on-the-go with the Contigo Autoseal West Loop 16 oz. This compact stainless steel bottle is a lid-because-you'll-never-spill-it gem, thanks to its Autoseal technology. Double-wall insulation keeps drinks hot or cold for hours. Take it to the gym, office, or park - this bottle's got you covered. Plus, its lifetime warranty gives you peace of mind. Pour yourself a fresh drink with confidence, knowing your bottle can keep up with your active lifestyle.</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>8484</v>
+      </c>
+      <c r="G26" t="n">
+        <v>192</v>
+      </c>
+      <c r="H26" t="n">
+        <v>105</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nike Air Zoom Pegasus 40</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>features: React foam, Zoom Air units, engineered mesh upper; energy efficient</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>textile &amp; synthetic</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2-year manufacturer warranty</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Take your runs to the next level with the Nike Air Zoom Pegasus 40. This sleek and lightweight shoe is designed for maximum comfort and performance. The React foam midsole and Zoom Air units provide a springy, energy-efficient ride, while the engineered mesh upper breathes easily to keep you cool and dry. With a 2-year manufacturer warranty, you can trust this shoe to last. Get ready to crush your fitness goals with the Pegasus 40 - perfect for runners of all levels.</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6885</v>
+      </c>
+      <c r="G27" t="n">
+        <v>192</v>
+      </c>
+      <c r="H27" t="n">
+        <v>101</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Adidas Ultraboost Light</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>features: Light BOOST midsole, Primeknit+ upper, Continental rubber; rating: 4.7/5</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>textile &amp; synthetic</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2-year manufacturer warranty</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Experience the comfort and versatility of the Adidas Ultraboost Light. This sleek shoe boasts a Light Boost midsole for seamless energy return, while the Primeknit+ upper ensures a snug, sock-like fit. With Continental rubber for grip and durability, you're ready for anything from casual strolls to high-intensity workouts. Rated 4.7/5, this shoe has been praised by thousands. Trust in the Adidas quality, backed by a 2-year manufacturer warranty for added peace of mind. Take your everyday runs smoother with the Ultraboost Light.</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>8708</v>
+      </c>
+      <c r="G28" t="n">
+        <v>199</v>
+      </c>
+      <c r="H28" t="n">
+        <v>114</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>The North Face ThermoBall Eco Jacket</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>features: synthetic ThermoBall insulation, DWR finish; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>100% recycled nylon</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Stay warm and keep the planet green with The North Face ThermoBall Eco Jacket. This tech-savvy jacket boasts synthetic ThermoBall insulation that traps heat like down, while the DWR finish repels water. Made from 100% recycled nylon, you'll feel good about your gear. Plus, a compact design makes it easy to stash in your bag. And don't worry, it's backed by a lifetime warranty. Perfect for commuting or hitting the trails, this eco-friendly jacket combines performance and sustainability.</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>8348</v>
+      </c>
+      <c r="G29" t="n">
+        <v>192</v>
+      </c>
+      <c r="H29" t="n">
+        <v>105</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Patagonia Black Hole 32 L Backpack</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>features: weather-resistant, laptop sleeve, padded straps; capacity: large</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>100% recycled polyester ripstop</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Embark on any adventure with confidence and style in the Patagonia Black Hole 32L Backpack. Built to withstand the elements, this weather-resistant pack keeps your gear dry and protected. Designed for comfort, it boasts padded straps and a dedicated laptop sleeve. Crafted from 100% recycled polyester ripstop, it's tough and sustainable. Plus, you can count on a lifetime warranty to stand by your investment. Whether you're hiking, commuting, or exploring, this rugged companion has got your back.</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>8032</v>
+      </c>
+      <c r="G30" t="n">
+        <v>194</v>
+      </c>
+      <c r="H30" t="n">
+        <v>103</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Osprey Farpoint 40</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>features: stowaway harness, laptop sleeve, carry-on size; energy efficient</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>450D recycled nylon</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Elevate your travels with the Osprey Farpoint 40. This versatile backpack seamlessly transitions from hiking trail to airport terminal, featuring a stowaway harness and laptop sleeve for streamlined carry-ons. Durable 450D recycled nylon withstands the rigors of adventure travel. Plus, with our lifetime warranty, you can trust this pack to keep up with your ever-changing itinerary. Reduce your footprint on the go with Osprey's energy-efficient design, built to keep you moving and exploring responsibly.</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>7653</v>
+      </c>
+      <c r="G31" t="n">
+        <v>192</v>
+      </c>
+      <c r="H31" t="n">
+        <v>103</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LEGO Star Wars Millennium Falcon 75192</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>features: 7 541 pieces, detailed interior, minifigs included; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ABS plastic bricks</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>lifetime replacement of missing bricks</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Get ready to embark on an epic adventure with the ultimate LEGO Star Wars experience! The Millennium Falcon 75192 is the most detailed and impressive set ever created, featuring an astonishing 7,541 pieces. With a richly detailed interior and 7 minifigures, this iconic spaceship comes to life in your hands. Built to last with high-quality ABS plastic bricks, this set is designed to withstand even the most intense play. And with a lifetime warranty, you can create and play without worry. May the force be with you!</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>7395</v>
+      </c>
+      <c r="G32" t="n">
+        <v>198</v>
+      </c>
+      <c r="H32" t="n">
+        <v>109</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LEGO Icons Botanical Orchid 10311</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>features: 608 pieces, adjustable blooms, decorative set; color options: multiple</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ABS plastic bricks</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>lifetime replacement of missing bricks</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Create a stunning centerpiece with the LEGO Icons Botanical Orchid 10311! This 608-piece decorative set lets you customize the blooms to your taste, with multiple color options to match your unique style. Made from high-quality ABS plastic bricks, this beautiful orchid is built to last. Plus, with our lifetime replacement warranty, you can enjoy your gorgeous flower for years to come. Perfect for plant lovers and LEGO enthusiasts alike, this set is a must-have for any room.</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>6377</v>
+      </c>
+      <c r="G33" t="n">
+        <v>195</v>
+      </c>
+      <c r="H33" t="n">
+        <v>97</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Kindle Paperwhite 11th Gen</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>features: 6.8″ glare-free display, 10-week battery, USB-C; dimensions: compact</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>recycled plastic</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Immerse yourself in your favorite stories with the Kindle Paperwhite 11th Gen. Its 6.8" glare-free display brings words to life in a distraction-free environment, while its 10-week battery keeps you reading all night long. Compact and portable, you can take it anywhere. Built with 30% recycled plastic, you can read with a clear conscience. The 1-year limited warranty gives you peace of mind. Upgrade your reading experience with this sleek and sustainable device that's designed to bring you and your books together.</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>8168</v>
+      </c>
+      <c r="G34" t="n">
+        <v>198</v>
+      </c>
+      <c r="H34" t="n">
+        <v>110</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Kobo Libra 2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>features: 7″ E Ink Carta, Bluetooth audiobooks, waterproof IPX8; weight: light</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>plastic chassis</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Meet your new travel companion: the Kobo Libra 2! This sleek and lightweight e-reader boasts a stunning 7" E Ink Carta display, making text crisp and clear in any light. Enjoy seamless audiobook playback via Bluetooth and dive into your favorite stories with confidence - it's waterproof, too! Weighing in at a mere x oz, this compact device fits easily in your bag and is built to last with a 1-year limited warranty for peace of mind. Discover a new way to read with Kobo Libra 2.</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>7697</v>
+      </c>
+      <c r="G35" t="n">
+        <v>198</v>
+      </c>
+      <c r="H35" t="n">
+        <v>113</v>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Anker Soundcore Motion+ Speaker</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>features: 30 W audio, Hi-Res, IPX7 waterproof; energy efficient</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>aluminum grille</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>18-month warranty</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>"Take your music anywhere with the Anker Soundcore Motion+ Speaker! Powerful 30W audio delivers crisp, Hi-Res sound that's sure to impress. Don't worry about water droplets - this speaker is IPX7 waterproof, so you can enjoy your tunes by the pool or on a rainy day. The durable aluminum grille ensures a premium build, while energy efficiency keeps you going all day. Backed by an 18-month warranty, this speaker is a reliable companion for any music lover on-the-go!"</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>7049</v>
+      </c>
+      <c r="G36" t="n">
+        <v>193</v>
+      </c>
+      <c r="H36" t="n">
+        <v>106</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sonos Move 2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>features: WiFi &amp; Bluetooth, 24-hr battery, automatic Trueplay; rating: 4.7/5</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>shock-resistant shell</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>"Take your music anywhere with the Sonos Move 2! This waterproof and shock-resistant powerhouse boasts a 24-hour battery life, rocking out all day and night. Automatic Trueplay fine-tunes sound to your space, ensuring crystal-clear highs and thumping lows. Stream effortlessly via WiFi or Bluetooth, and enjoy peace of mind with a 4.7/5 rating and 1-year limited warranty. Unplug, untether, and lose yourself in your favorite tunes – the perfect companion for outdoor adventures and indoor vibes alike!"</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>6970</v>
+      </c>
+      <c r="G37" t="n">
+        <v>199</v>
+      </c>
+      <c r="H37" t="n">
+        <v>108</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Philips Hue White &amp; Color Ambiance Starter Kit</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>features: 16 million colors, Bluetooth &amp; Zigbee, voice control; limited edition</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>plastic bulbs</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Elevate your home's ambiance with Philips Hue's innovative Starter Kit. This limited-edition collection features 16 million colors, blending seamlessly into any space. With voice control and wireless connectivity via Bluetooth and Zigbee, you can effortlessly adjust the atmosphere. Our durable plastic bulbs ensure long-lasting performance, and our 2-year limited warranty provides peace of mind. Unleash endless color possibilities and rediscover the joy of lights that transform with you.</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>5732</v>
+      </c>
+      <c r="G38" t="n">
+        <v>195</v>
+      </c>
+      <c r="H38" t="n">
+        <v>91</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TP-Link Deco XE75 Mesh WiFi 6E</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>features: tri-band AXE5400, 3-pack covers 7 200 sq ft; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Expand your WiFi coverage with the TP-Link Deco XE75, a powerful 3-pack mesh system that blankets up to 7,200 sq ft with strong, reliable connections. Enjoy seamless streaming and gaming on your latest devices with its tri-band AXE5400 technology. And with long-lasting batteries, setup and maintenance are a breeze. Backed by a 2-year limited warranty, this device keeps you connected with confidence. Invest in a resilient and lag-free WiFi experience, free from dead zones and dropped connections. Stay connected.</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>7080</v>
+      </c>
+      <c r="G39" t="n">
+        <v>205</v>
+      </c>
+      <c r="H39" t="n">
+        <v>110</v>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Eufy Video Doorbell Dual</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>features: dual camera, package detection, 2K resolution; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>plastic housing</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>"Stay safe and sound with the Eufy Video Doorbell Dual. This cutting-edge doorbell features two cameras for crystal-clear 2K resolution, so you never miss a visitor. Its intelligent package detection alerts you to deliveries or potential threats, giving you peace of mind. With long-lasting battery life and a durable plastic housing, this doorbell is designed to last. Plus, you're protected by a 1-year limited warranty. Keep your home secure and connected with the Eufy Video Doorbell Dual."</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>5818</v>
+      </c>
+      <c r="G40" t="n">
+        <v>193</v>
+      </c>
+      <c r="H40" t="n">
+        <v>105</v>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Blink Outdoor 4</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>features: 1080p HD, 2-year battery, weather-resistant; limited edition</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Enhance your home security with the limited edition Blink Outdoor 4. This versatile camera boasts 1080p HD video, ensuring crystal-clear footage, day or night. Durable and weather-resistant, it withstands the elements with ease, while its 2-year battery and simple wire-free setup make it effortless to install. As a limited edition, this secure home accessory is a rare find. Protect what matters most with a 1-year limited warranty and the confidence that comes with unparalleled night vision.</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>24238</v>
+      </c>
+      <c r="G41" t="n">
+        <v>190</v>
+      </c>
+      <c r="H41" t="n">
+        <v>101</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Corsair K100 RGB Keyboard</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>features: Cherry MX Speed, 4000 Hz polling, aluminum frame; capacity: large</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>brushed aluminum</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2-year warranty</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Elevate your gaming experience with the Corsair K100 RGB Keyboard. This powerhouse features Cherry MX Speed switches for lightning-fast actuation and 4000 Hz polling for seamless communication with your computer. The rugged aluminum frame withstands heavy use, while the large capacity layout provides ample space for your fingers to roam. Experience unparalleled performance and precision, backed by a 2-year warranty that gives you peace of mind. Upgrade your setup today and take your gaming to the next level!</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>8421</v>
+      </c>
+      <c r="G42" t="n">
+        <v>192</v>
+      </c>
+      <c r="H42" t="n">
+        <v>97</v>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Logitech MX Master 3S</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>features: 8K DPI sensor, MagSpeed scroll, Bolt &amp; Bluetooth; color options: multiple</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Elevate your workspace with the Logitech MX Master 3S, expertly designed for professionals on the go. This ergonomic mouse boasts an astonishing 8K DPI sensor for precise tracking, plus MagSpeed scroll for lightning-fast navigation. Connect via Bolt, Bluetooth, or multiple color options to match your style. The durable plastic construction withstands daily use, and a 1-year limited warranty gives you peace of mind. Upgrade your productivity with confidence and exceptional performance.</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>10246</v>
+      </c>
+      <c r="G43" t="n">
+        <v>195</v>
+      </c>
+      <c r="H43" t="n">
+        <v>95</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Razer DeathAdder V3 Pro</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>features: 63 g ultralight, 30K DPI Focus Pro sensor; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2-year warranty</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Level up your gaming experience with the Razer DeathAdder V3 Pro! This ultralight champion (just 63g) lets you move fast and stay focused on the mission. The 30K DPI Focus Pro sensor delivers lightning-quick accuracy, while the long-lasting battery ensures you can play on for hours without interruption. Built with precision plastic, this mouse is designed to last, with a 2-year warranty to back it up. Get ready to dominate the competition with the DeathAdder V3 Pro - the ultimate gaming companion.</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>18080</v>
+      </c>
+      <c r="G44" t="n">
+        <v>196</v>
+      </c>
+      <c r="H44" t="n">
+        <v>111</v>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Samsung 980 Pro 2 TB NVMe SSD</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>features: PCIe 4.0, up to 7 000 MB/s read, nickel coating; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PCB &amp; NAND flash</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>5-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Level up your storage game with the Samsung 980 Pro 2 TB NVMe SSD! Powered by PCIe 4.0, this blazing-fast drive boasts read speeds of up to 7,000 MB/s, ensuring seamless multitasking and lightning-quick loading times. With its long-lasting battery and rugged nickel coating, this SSD is built to last. Backed by a 5-year limited warranty, you can trust it to keep up with your demanding needs. Upgrade your PC with the best - get the Samsung 980 Pro today!</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>7978</v>
+      </c>
+      <c r="G45" t="n">
+        <v>206</v>
+      </c>
+      <c r="H45" t="n">
+        <v>109</v>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Seagate Portable 5 TB HDD</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>features: USB 3.0, plug-and-play, 2.5″ form factor; rating: 4.7/5</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>plastic shell</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1-year limited warranty</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Expand your storage capacity with the Seagate Portable 5 TB HDD, a reliable and convenient solution. This plug-and-play external hard drive features USB 3.0 connectivity, allowing for fast data transfer speeds. The compact 2.5" form factor makes it perfect for laptops or desktops, while the tough plastic shell ensures durability. With a 4.7/5 rating, thousands have already trusted this hard drive to safeguard their digital files. Backed by a 1-year limited warranty, you can enjoy peace of mind.</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>6935</v>
+      </c>
+      <c r="G46" t="n">
+        <v>204</v>
+      </c>
+      <c r="H46" t="n">
+        <v>109</v>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SanDisk Extreme PRO 128 GB SDXC</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>features: UHS-I U3, 200 MB/s read, waterproof; battery: long-lasting</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>lifetime limited warranty</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>"Capture life's most epic moments with the SanDisk Extreme PRO 128 GB SDXC! This rugged card features blazing-fast UHS-I U3 transfers at 200 MB/s, so you can quickly offload your shots. Plus, it's waterproof, so you don't have to worry about accidental spills or ocean encounters. With a long-lasting battery life, you'll be able to shoot all day without worrying about running out of juice. Get the peace of mind and flexibility you need to take your photography to the next level!"</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>8252</v>
+      </c>
+      <c r="G47" t="n">
+        <v>195</v>
+      </c>
+      <c r="H47" t="n">
+        <v>108</v>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Kingston Fury Beast 32 GB DDR5</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>features: 6000 MT/s, Intel XMP 3.0, low-profile heat spreader; energy efficient</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>aluminum heatspreader</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>lifetime warranty</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Boost your gaming and performance with the Kingston Fury Beast 32 GB DDR5 memory kit! With speeds of 6000 MT/s, you'll enjoy responsive and immersive experiences. Featuring Intel XMP 3.0 and a low-profile heat spreader, this kit keeps your system running smoothly. Plus, its energy-efficient design and aluminum heatspreader ensure reliable performance and extended lifespan. Rely on the Fury Beast's lifetime warranty and unlock your full gaming potential - upgrade today!</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>7183</v>
+      </c>
+      <c r="G48" t="n">
+        <v>200</v>
+      </c>
+      <c r="H48" t="n">
+        <v>97</v>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Acer Predator XB273U 27″ Monitor</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>features: 2560*1440 170 Hz IPS, HDR400, G-Sync Compatible; capacity: large</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>plastic &amp; metal stand</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>3-year warranty</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Get ready to take your gaming and graphic design to the next level with the Acer Predator XB273U 27" Monitor! Enjoy stunning visuals with its 2560*1440 170Hz IPS display, HDR400 capabilities, and seamless G-Sync Compatible performance. The large screen and reliable 3-year warranty give you the confidence to push your creative limits. Plus, the durable plastic and metal stand keeps this beast stable on your desk. Upgrade your workflow today and experience the power of precision!</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>6225</v>
+      </c>
+      <c r="G49" t="n">
+        <v>203</v>
+      </c>
+      <c r="H49" t="n">
+        <v>101</v>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BenQ PD2725U 27″ Monitor</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>features: 4K UHD IPS, 98% P3, Thunderbolt 3; color options: multiple</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>metal stand</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>3-year warranty</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Elevate your creative workflow with the BenQ PD2725U monitor. Effortlessly view lifelike colors and precise details on its 4K UHD IPS display, covering a wide 98% of the P3 color space. Transfer files and collaborate seamlessly with Thunderbolt 3 connectivity. Choose from multiple color options to match your unique style. Enjoy peace of mind with a 3-year warranty. Upgrade your visual experience and unlock your full creative potential with this expert-grade display.</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>6201</v>
+      </c>
+      <c r="G50" t="n">
+        <v>202</v>
+      </c>
+      <c r="H50" t="n">
+        <v>101</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ASUS ProArt PA278QV Monitor</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>features: 27″ 2560*1440 IPS, 100% sRGB, Calman Verified; weight: light</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>metal stand</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>3-year warranty</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Unlock your creative potential with the ASUS ProArt PA278QV Monitor. This stunning 27" display boasts vibrant colors in crisp 2560x1440 resolution, ensuring every detail pops. With 100% sRGB coverage, you can trust the accuracy of your work. The Calman Verified certification guarantees precise color representation. Built to last, the monitor's sleek metal stand is both lightweight and durable, while a 3-year warranty gives you peace of mind. Experience unparalleled picture quality and unleash your artistry with this exceptional display.</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>6597</v>
+      </c>
+      <c r="G51" t="n">
+        <v>202</v>
+      </c>
+      <c r="H51" t="n">
+        <v>109</v>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Jupyter notebook with cost calculation improvements and execution count adjustments
- Updated execution counts for code cells to reflect the latest execution order.
- Refactored cost calculation logic to improve clarity and consistency in variable naming.
- Added functionality to save results to an Excel file after calculations.
</commit_message>
<xml_diff>
--- a/assignment_01.xlsx
+++ b/assignment_01.xlsx
@@ -539,7 +539,9 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>1.048e-05</v>
+      </c>
       <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -583,7 +585,9 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>1.078e-05</v>
+      </c>
       <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -627,7 +631,9 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>1.058e-05</v>
+      </c>
       <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -671,7 +677,9 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="n">
+        <v>1.098e-05</v>
+      </c>
       <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -715,7 +723,9 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="n">
+        <v>1.078e-05</v>
+      </c>
       <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -759,7 +769,9 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="n">
+        <v>1.038e-05</v>
+      </c>
       <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -803,7 +815,9 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="n">
+        <v>1.092e-05</v>
+      </c>
       <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -847,7 +861,9 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" t="n">
+        <v>9.820000000000001e-06</v>
+      </c>
       <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -891,7 +907,9 @@
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="n">
+        <v>1.024e-05</v>
+      </c>
       <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -935,7 +953,9 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="n">
+        <v>1.02e-05</v>
+      </c>
       <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -979,7 +999,9 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="n">
+        <v>1.04e-05</v>
+      </c>
       <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1023,7 +1045,9 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="n">
+        <v>1.02e-05</v>
+      </c>
       <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1067,7 +1091,9 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="n">
+        <v>1.096e-05</v>
+      </c>
       <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1111,7 +1137,9 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="n">
+        <v>1.006e-05</v>
+      </c>
       <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1155,7 +1183,9 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="n">
+        <v>9.840000000000001e-06</v>
+      </c>
       <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1199,7 +1229,9 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="O17" t="n">
+        <v>1.028e-05</v>
+      </c>
       <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1243,7 +1275,9 @@
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="O18" t="n">
+        <v>1.15e-05</v>
+      </c>
       <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1287,7 +1321,9 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" t="n">
+        <v>1.024e-05</v>
+      </c>
       <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1331,7 +1367,9 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" t="n">
+        <v>9.76e-06</v>
+      </c>
       <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1375,7 +1413,9 @@
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="n">
+        <v>9.94e-06</v>
+      </c>
       <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1419,7 +1459,9 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="n">
+        <v>9.72e-06</v>
+      </c>
       <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1463,7 +1505,9 @@
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="n">
+        <v>9.96e-06</v>
+      </c>
       <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1507,7 +1551,9 @@
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" t="n">
+        <v>1.02e-05</v>
+      </c>
       <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1551,7 +1597,9 @@
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="n">
+        <v>9.299999999999999e-06</v>
+      </c>
       <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1595,7 +1643,9 @@
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="n">
+        <v>1.014e-05</v>
+      </c>
       <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1639,7 +1689,9 @@
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="n">
+        <v>9.9e-06</v>
+      </c>
       <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1683,7 +1735,9 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="O28" t="n">
+        <v>1.082e-05</v>
+      </c>
       <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1727,7 +1781,9 @@
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="O29" t="n">
+        <v>1.014e-05</v>
+      </c>
       <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1771,7 +1827,9 @@
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
+      <c r="O30" t="n">
+        <v>1.006e-05</v>
+      </c>
       <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1815,7 +1873,9 @@
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="O31" t="n">
+        <v>1.002e-05</v>
+      </c>
       <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1859,7 +1919,9 @@
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" t="n">
+        <v>1.05e-05</v>
+      </c>
       <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1903,7 +1965,9 @@
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="n">
+        <v>9.72e-06</v>
+      </c>
       <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1947,7 +2011,9 @@
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" t="n">
+        <v>1.056e-05</v>
+      </c>
       <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1991,7 +2057,9 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" t="n">
+        <v>1.074e-05</v>
+      </c>
       <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -2035,7 +2103,9 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="n">
+        <v>1.022e-05</v>
+      </c>
       <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2079,7 +2149,9 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="n">
+        <v>1.046e-05</v>
+      </c>
       <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -2123,7 +2195,9 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="O38" t="n">
+        <v>9.36e-06</v>
+      </c>
       <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -2167,7 +2241,9 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="n">
+        <v>1.07e-05</v>
+      </c>
       <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2211,7 +2287,9 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="O40" t="n">
+        <v>1.016e-05</v>
+      </c>
       <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2255,7 +2333,9 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="n">
+        <v>9.86e-06</v>
+      </c>
       <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2299,7 +2379,9 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="O42" t="n">
+        <v>9.659999999999999e-06</v>
+      </c>
       <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2343,7 +2425,9 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="n">
+        <v>9.6e-06</v>
+      </c>
       <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -2387,7 +2471,9 @@
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="O44" t="n">
+        <v>1.058e-05</v>
+      </c>
       <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
@@ -2431,7 +2517,9 @@
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="O45" t="n">
+        <v>1.066e-05</v>
+      </c>
       <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2475,7 +2563,9 @@
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
+      <c r="O46" t="n">
+        <v>1.062e-05</v>
+      </c>
       <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2519,7 +2609,9 @@
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
+      <c r="O47" t="n">
+        <v>1.038e-05</v>
+      </c>
       <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2563,7 +2655,9 @@
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="O48" t="n">
+        <v>9.820000000000001e-06</v>
+      </c>
       <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
@@ -2607,7 +2701,9 @@
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
+      <c r="O49" t="n">
+        <v>1.012e-05</v>
+      </c>
       <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
@@ -2651,7 +2747,9 @@
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="O50" t="n">
+        <v>1.01e-05</v>
+      </c>
       <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2695,7 +2793,9 @@
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="O51" t="n">
+        <v>1.058e-05</v>
+      </c>
       <c r="P51" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ran task 4 experiment 1 after refactoring notebook for easy reuse
</commit_message>
<xml_diff>
--- a/assignment_01.xlsx
+++ b/assignment_01.xlsx
@@ -531,23 +531,23 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Get ready to take your mobile experience to the next level with the Apple iPhone 15 Pro! Powered by the lightning-fast A17 Pro chip, this powerhouse of a phone delivers instant response times and seamless performance. The stunning 120 Hz ProMotion display boasts vibrant colors and silky-smooth visuals. Enjoy fast and convenient charging via USB-C, and rest assured with a 1-year limited warranty. Plus, its compact design makes it effortless to carry, all wrapped up in a durable titanium frame and tough Ceramic Shield glass.</t>
+          <t>Take your mobile experience to the next level with the iPhone 15 Pro. Powered by the lightning-fast A17 Pro chip, this powerhouse seamlessly navigates demanding tasks and tasks with ease. A stunning 120 Hz ProMotion display ensures a buttery-smooth visuals. Plus, enjoy quick refueling with fast USB-C charging. Built with a strong titanium frame and Ceramic Shield glass for added durability, this compact phone is as rugged as it is refined. Sensational performance meets luxury build quality – elevate your daily life with the iPhone 15 Pro.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3475</v>
+        <v>4720</v>
       </c>
       <c r="G2" t="n">
         <v>200</v>
       </c>
       <c r="H2" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I2" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="J2" t="n">
-        <v>1.03e-05</v>
+        <v>1.06e-05</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -613,23 +613,23 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Elevate your mobile experience with the Samsung Galaxy S24 Ultra. This powerhouse phone boasts a 200 MP camera, allowing you to capture stunning details and vibrant colors. The S-Pen supports note-taking, drawing, and more, while the seamless 120 Hz AMOLED display provides an immersive viewing experience. Sourced responsibly from the earth, this sleek device also features a durable Armor Aluminum frame and scratch-resistant Gorilla Glass Victus. Enjoy peace of mind with a 1-year limited warranty. Unlock new possibilities with the Galaxy S24 Ultra.</t>
+          <t>Upgrade your mobile experience with the Samsung Galaxy S24 Ultra. This powerhouse features a 200 MP camera that captures stunning detail, plus S-Pen support for notebook-esque notes and creative freedom. The 120 Hz AMOLED display is silky smooth, while the Armor Aluminum frame and Gorilla Glass Victus ensure durability. Plus, Samsung's commitment to sustainability means peace of mind with every use. Backed by a 1-year limited warranty, this phone is built to last and perform. Unlock endless possibilities with the Galaxy S24 Ultra.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6270</v>
+        <v>3671</v>
       </c>
       <c r="G3" t="n">
         <v>203</v>
       </c>
       <c r="H3" t="n">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="I3" t="n">
         <v>83</v>
       </c>
       <c r="J3" t="n">
-        <v>1.078e-05</v>
+        <v>1.06e-05</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -695,23 +695,23 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>"Unlock a world of breathtaking photography with the Google Pixel 8 Pro. Powered by the advanced Tensor G3 chip, this powerhouse camera phone captures life's moments with precision and clarity. With the innovative Magic Eraser, unwanted objects vanish in an instant. Featuring a 50 MP camera and a stunning 4.7/5 rating, this device is a must-have for smartphone enthusiasts. Enjoy a premium design in matte glass and aluminum, backed by a 1-year limited warranty for added peace of mind."</t>
+          <t>"Unlock the future of smartphone photography with the Google Pixel 8 Pro. Powered by the innovative Tensor G3 chip, this flagship device delivers unparalleled performance and results. The 50 MP camera, paired with Magic Eraser technology, lets you erase unwanted objects from your photos with a single tap. With a 4.7/5 rating and a 1-year warranty, you can trust the Pixel 8 Pro to capture life's precious moments and last. Its stunning design, featuring a matte glass back and aluminum frame, makes it a stunning addition to any style."</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3611</v>
+        <v>3210</v>
       </c>
       <c r="G4" t="n">
         <v>202</v>
       </c>
       <c r="H4" t="n">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="I4" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="J4" t="n">
-        <v>1.022e-05</v>
+        <v>1.094e-05</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -777,23 +777,23 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Escape to serenity with the Sony WH-1000XM5 Headphones. Powered by industry-leading active noise cancelling, these headphones transport you to a world of tranquility, blocking out distractions and immersing you in crystal-clear sound. Enjoy up to 30 hours of wireless freedom, recharging quickly via Bluetooth 5.2. Premium synthetic leather earcups cradle your ears in comfort. Backed by a 1-year limited warranty, you can rely on these exceptional headphones to elevate your daily commutes, workouts, or relaxation sessions.</t>
+          <t>"Immerse yourself in pure sound with the Sony WH-1000XM5 Headphones! These powerful cans deliver uncompromising audio, instant noise cancellation, and seamless connectivity via Bluetooth 5.2. Enjoy up to 30 hours of listening without a break. The large capacity and sleek design ensure a comfortable fit. Durable synthetic leather earcups provide long-lasting durability. Protect your investment with a 1-year limited warranty. Perfect for music lovers, commuters, and anyone seeking exceptional audio on-the-go."</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3896</v>
+        <v>3309</v>
       </c>
       <c r="G5" t="n">
         <v>201</v>
       </c>
       <c r="H5" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="I5" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J5" t="n">
-        <v>1.074e-05</v>
+        <v>1.038e-05</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -859,23 +859,23 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Transform your music experience with the Bose QuietComfort Ultra Earbuds! These award-winning earbuds deliver a personalized sound that adapts to your unique hearing, thanks to CustomTune sound calibration. Enjoy immersive listening freedom with Advanced Noise Cancellation (ANC) and stay active with IPX4 sweat and water resistance. Plus, comfortable silicone ear tips ensure all-day wearing. With a 1-year limited warranty, you can trust your new earbuds to perform. Upgrade your music moments – try the QuietComfort Ultra Earbuds today!</t>
+          <t>Immerse yourself in crystal-clear audio with the Bose QuietComfort Ultra Earbuds. These sleek earbuds deliver tailored sound through CustomTune calibration, ensuring you hear every note as it was meant to be. Advanced Noise Cancellation blocks out distractions, while IPX4 protection keeps them safe from the elements. With an award-winning design and comfortable silicone ear tips, you'll enjoy hours of uninterrupted listening - anywhere, anytime. Backed by a one-year warranty, these earbuds are an investment in your listening experience.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4041</v>
+        <v>3637</v>
       </c>
       <c r="G6" t="n">
         <v>194</v>
       </c>
       <c r="H6" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I6" t="n">
         <v>78</v>
       </c>
       <c r="J6" t="n">
-        <v>1.048e-05</v>
+        <v>1.036e-05</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -941,23 +941,23 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>"Elevate your home with the Amazon Echo Dot (5th Gen), a sophisticated smart speaker that seamlessly blends form and function. With Alexa's voice assistant, you can control your space with effortless ease. The improved bass and temperature sensor ensure an immersive listening experience, while the sustainably sourced mesh fabric exudes an eco-friendly charm. Plus, with a 1-year limited warranty, you can relax knowing you're protected. Upgrade your smart setup with the Echo Dot and experience the perfect blend of sound and style."</t>
+          <t>Get ready to elevate your smart home experience with the Amazon Echo Dot (5th Gen). This groundbreaking device boasts an improved Alexa voice assistant, so you can control your smart devices with just your voice. Add to that, an integrated temperature sensor and enhanced bass for a richer audio experience. Plus, it's wrapped in sustainable, recycled fabric mesh and backed by a 1-year limited warranty. Upgrade your space with the perfect blend of tech and eco-friendliness.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3167</v>
+        <v>3316</v>
       </c>
       <c r="G7" t="n">
         <v>192</v>
       </c>
       <c r="H7" t="n">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="I7" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="J7" t="n">
-        <v>1.008e-05</v>
+        <v>9.480000000000001e-06</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1023,23 +1023,23 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Upgrade your productivity with the Dell XPS 13 9310 laptop, designed for modern professionals on the go. Its compact CNC aluminum and carbon-fiber palmrest build ensures a durable and sleek design. The 13.4" FHD+ display provides vibrant visuals, while the Intel Core i5 processor handles demanding tasks with ease. With Thunderbolt 4 connectivity and a 1-year limited hardware warranty, you can work with confidence. Stay ahead of the curve with this powerful and portable workstation.</t>
+          <t>Meet the Dell XPS 13 9310, the ultimate travel companion! This stunning laptop packs a 13.4" FHD+ display and lightning-fast Intel Core i5 processor, perfect for work, play, and everything in between. Its compact design and durable CNC aluminum and carbon-fiber palmrest ensure it withstands even the toughest handbags. With Thunderbolt 4 and reliable 1-year limited hardware warranty, you can stay productive and confident on-the-go. Upgrade your mobile game with this fantastic device and experience the bliss of seamless performance!</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3375</v>
+        <v>2824</v>
       </c>
       <c r="G8" t="n">
         <v>210</v>
       </c>
       <c r="H8" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="I8" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="J8" t="n">
-        <v>1.032e-05</v>
+        <v>1.104e-05</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1105,23 +1105,23 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Take your productivity on the go with the Apple MacBook Air 13". Powered by the efficient M3 chip, this ultraportable laptop delivers all-day battery life - up to 18 hours of non-stop performance. Plus, its 1080p camera ensures crisp, clear video chats. The durable recycled aluminum unibody construction withstands daily wear and tear. Protected by a 1-year limited warranty, this reliable machine is your perfect companion for work, play, and everything in between. Experience the ultimate in portability and power.</t>
+          <t>Take your creativity to new heights with the Apple MacBook Air 13". Powered by the lightning-fast M3 chip, you'll experience seamless performance and effortless multitasking. With up to 18 hours of battery life, you can work, create, and play all day without interruptions. Plus, a 1080p camera lets you connect with friends and family in crystal-clear video calls. Crafted from durable recycled aluminum, this eco-conscious laptop combines style and sustainability.</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4892</v>
+        <v>2103</v>
       </c>
       <c r="G9" t="n">
         <v>200</v>
       </c>
       <c r="H9" t="n">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="I9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J9" t="n">
-        <v>1.06e-05</v>
+        <v>9.639999999999999e-06</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1187,23 +1187,23 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Unlock the ultimate productivity experience! The Microsoft Surface Pro 10 boasts a powerful Intel Core Ultra processor, paired with a stunning 13" PixelSense touchscreen. Easily detach the keyboard and take your work on the go with this ultra-compact, magnesium alloy chassis design. Plus, enjoy the peace of mind that comes with our 1-year limited warranty. Whether you create, work, or play, this laptop Substitute redefines mobile flexibility, empowering you to stay ahead of the curve, anywhere, anytime.</t>
+          <t>Get ready to upgrade your productivity on the go with the Microsoft Surface Pro 10! This powerful tablet boasts the latest Intel Core Ultra processor, effortlessly running multiple apps and tasks with ease. With a stunning 13" PixelSense display and detachable keyboard, you can switch seamlessly between laptop and tablet modes. Made from sturdy magnesium alloy, this compact device is both durable and stylish. Enjoy worry-free computing with a 1-year limited warranty - buy with confidence and take your mobile work to the next level!</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5746</v>
+        <v>2358</v>
       </c>
       <c r="G10" t="n">
         <v>194</v>
       </c>
       <c r="H10" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I10" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="J10" t="n">
-        <v>9.94e-06</v>
+        <v>9.999999999999999e-06</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1269,23 +1269,23 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Take your running to new heights with the Garmin Forerunner 255! This sleek, fiber-reinforced device guides you with multi-band GPS, tracking every detail of your performance. Get a deeper understanding of your body's stress levels with HRV status. Enjoy up to 14 days on a single charge, all while shaving grams of weight. Join the thousands who've rated it 4.7/5! With a 1-year limited warranty, you can trust your purchase. Join the Forerunner family and unlock your full potential today!</t>
+          <t>Take your running to the next level with the Garmin Forerunner 255. Boasting a robust multi-band GPS, this watch provides accurate tracking and location data, even in the most rugged terrain. Plus, with HRV status, you'll receive advanced insights into your physical condition. And with up to 14 days of battery life, you can track your run without worrying about running out of juice. Get ready to crush your personal records with this reliable and feature-packed companion.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3981</v>
+        <v>2377</v>
       </c>
       <c r="G11" t="n">
         <v>201</v>
       </c>
       <c r="H11" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J11" t="n">
-        <v>1.074e-05</v>
+        <v>9.840000000000001e-06</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1351,21 +1351,21 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Take control of your fitness journey with the Fitbit Charge 6! This sleek and reliable tracker keeps pace with your active lifestyle, monitoring your heart rate in real-time and navigating your routes with built-in GPS. Enjoy up to 7 days of battery life on a single charge, and customize your look with multiple color options. Built with a sturdy aluminum case, this device is built to last. Plus, a 1-year limited warranty gives you peace of mind. Get fit, feel great, and achieve your goals with the Fitbit Charge 6.</t>
+          <t>Take your fitness journey to the next level with the Fitbit Charge 6! This sleek and durable wearable tracks your progress like a pro, featuring a heart-rate monitor and built-in GPS to log your runs, hikes, and workouts with ease. With up to 7 days of battery life, you can track your progress without worrying about running out of power. Choose from multiple vibrant color options to match your unique style. Get precise and stay motivated – order your Fitbit Charge 6 today and start achieving your fitness goals!</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3913</v>
+        <v>3061</v>
       </c>
       <c r="G12" t="n">
         <v>193</v>
       </c>
       <c r="H12" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
-        <v>1.058e-05</v>
+        <v>1.022e-05</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
@@ -1399,21 +1399,21 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>"Take your adventures to new heights with the GoPro HERO12 Black! Capture stunning 5.3K60 video and enjoy seamless stabilization with HyperSmooth 6.0, ensuring every shot is rock-solid. Intrepid explorers, rejoice – this rugged camera is waterproof up to 10m! Crafted from impact-resistant polycarbonate, it can withstand the toughest conditions. Trust in a 1-year limited warranty to back your purchase. Whether you're scaling mountains or diving into the unknown, the GoPro HERO12 Black is your ultimate visual partner."</t>
+          <t>Capture life's most epic moments with the GoPro HERO12 Black! This rugged adventure camera shoots stunning 5.3K60 video, ensuring thrilling footage every time. With HyperSmooth 6.0 stabilization, your videos will be silky-smooth even in turbulent conditions. Diving into the ocean? No problem - it's waterproof up to 10 meters! Built with a large capacity, this rugged polycarbonate housing can withstand extreme environments. Protected by a 1-year limited warranty, you can focus on the thrill of capturing life's unforgettable experiences.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>4837</v>
+        <v>3514</v>
       </c>
       <c r="G13" t="n">
         <v>201</v>
       </c>
       <c r="H13" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>1.086e-05</v>
+        <v>1.08e-05</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -1447,21 +1447,21 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Take your aerial adventures to new heights with the DJI Mini 4 Pro Drone! Weighing in at just under 250g, this compact powerhouse captures breathtaking 4K/60fps footage with ease. With advanced omnidirectional obstacle sensing, you'll navigate through complex environments with confidence. This top-rated drone (4.7/5) is built with durable composite plastic, ensuring a safe and reliable flying experience. Get ready to soar to new heights with DJI's flagship drone – your next aerial masterpiece awaits!</t>
+          <t>Capture life's most epic moments with the DJI Mini 4 Pro Drone! This powerhouse packs a 4K/60fps punch, letting you relive incredible memories in crystal-clear detail. Equipped with advanced omnidirectional obstacle sensing, you'll fly with confidence, even in confined spaces. Lightweight and versatile, this drone is perfect for pros and hobbyists alike. With a 4.7-star rating and a 1-year warranty, you can trust the quality and performance of this remarkable drone. Fly, capture, repeat!</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>5902</v>
+        <v>2997</v>
       </c>
       <c r="G14" t="n">
         <v>203</v>
       </c>
       <c r="H14" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
-        <v>1.048e-05</v>
+        <v>1.06e-05</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
@@ -1495,21 +1495,21 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Elevate your gaming experience with the Nintendo Switch OLED. This high-performance console boasts a stunning 7-inch OLED screen, providing crisp and vibrant visuals in both docked and handheld modes. With 64 GB of storage, you'll have ample room for your favorite games. The durable plastic chassis ensures a rugged build that can withstand the rigors of travel and play. Enjoy peace of mind with a 1-year limited warranty. Upgrade your gaming adventures today!</t>
+          <t>Elevate your gaming experience with the Nintendo Switch OLED. Boasting a vibrant 7″ OLED screen, this console delivers stunning visuals and immersive gameplay in both docked and handheld modes. With 64 GB of storage, you've got plenty of room to save all your favorite titles. Crafted with a durable plastic chassis, this console is built to last. And with a 1-year limited warranty, you can play with peace of mind. Get ready to take your gaming to the next level!</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>5406</v>
+        <v>2457</v>
       </c>
       <c r="G15" t="n">
         <v>194</v>
       </c>
       <c r="H15" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
-        <v>9.459999999999999e-06</v>
+        <v>9.999999999999999e-06</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -1543,21 +1543,21 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Get ready to take your gaming to the next level with the PlayStation 5 Slim! Experience immersive immersion with ray tracing and haptic feedback controller, putting you inside the action. A 1 TB SSD ensures seamless loading and quick access to your favorite games. Plus, the long-lasting battery keeps you gaming on the go. Wrapped in a durable plastic shell, you can count on it to perform. Enjoy 1-year of worry-free gaming with our limited warranty. Elevate your playtime, upgrade your console today!</t>
+          <t>Transform your gaming experience with the PlayStation 5 Slim! This sleek console boasts incredible features, including stunning ray tracing and an immersive haptic feedback controller. The 1 TB SSD ensures lightning-fast loading times, while the long-lasting battery gives you hours of uninterrupted fun. Wrapped in a durable plastic shell, this console is built to last. Your gaming world just got a serious upgrade - back it up with our 1-year limited warranty and take your gaming to the next level.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>8070</v>
+        <v>2520</v>
       </c>
       <c r="G16" t="n">
         <v>192</v>
       </c>
       <c r="H16" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>1.008e-05</v>
+        <v>9.6e-06</v>
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
@@ -1591,21 +1591,21 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Take your gaming experience to the next level with the Xbox Series X! This powerful console features a 12 TFLOPS GPU and 1 TB SSD, allowing for crisp 4K resolution at 120 Hz for ultra-smooth gameplay. Plus, its long-lasting battery keeps you gaming all day, every day. With a sleek matte black casing and 1-year limited warranty, you can keep up with the best gamers without breaking the bank. Upgrade now and get ready to experience unparalleled gaming performance!</t>
+          <t>"Unlock unparalleled gaming performance with the Xbox Series X, powered by a 12 TFLOPS GPU that brings stunning visuals to life at 4K and 120 frames per second. Enjoy seamless gameplay on the fast 1 TB SSD. The long-lasting battery keeps you gaming for hours. The sleek matte black casing is a stylish addition to any gaming setup. With a 1-year limited warranty, you can focus on what matters most - dominating on the gaming scene. Upgrade your gaming experience today with the Xbox Series X."</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>5848</v>
+        <v>6893</v>
       </c>
       <c r="G17" t="n">
         <v>199</v>
       </c>
       <c r="H17" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
-        <v>1.004e-05</v>
+        <v>1.034e-05</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -1639,21 +1639,21 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Take your cooking to the next level with the Instant Pot Duo 6-Quart! This versatile 7-in-1 multicooker simplifies meal prep with seven functions in one pot: pressure cooker, slow cooker, rice cooker, yogurt maker, sauté pan, and more. Built with a durable 18/8 stainless steel inner pot that's resistant to corrosion, and a lightweight design for easy maneuverability. 1000 W heating quickly gets you to your desired temperature. With a 1-year limited warranty, you can cook with confidence. Elevate your meals and enjoy cooking time savings!</t>
+          <t>Elevate your cooking experience with the versatile Instant Pot Duo 6-Quart! This 7-in-1 multicooker is a game-changer for home cooks. With its stainless steel inner pot and 1000 W heating, you can pressure cook, slow cook, sauté, steam, and more with ease. Plus, its lightweight design makes it easy to transfer between counters. Durable and built to last, the 18/8 stainless steel body and 1-year limited warranty ensure long-lasting reliability. Discover the power of a perfect meal, every time, with the Instant Pot Duo.</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>4278</v>
+        <v>4964</v>
       </c>
       <c r="G18" t="n">
         <v>206</v>
       </c>
       <c r="H18" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
-        <v>1.156e-05</v>
+        <v>1.162e-05</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -1687,21 +1687,21 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Elevate your coffee experience with the Keurig K-Supreme Plus Smart! This sleek and advanced brewer features multistream extraction technology, ensuring a perfect cup every time. The BrewID functionality connects you to your preferred coffee settings, making it easy to save and recall your favorite brews. With a large 78 oz reservoir and sleek brushed stainless steel accents, this machine is a must-have for any coffee connoisseur. Plus, enjoy peace of mind with a 1-year limited warranty. Upgrade your coffee routine today!</t>
+          <t>Elevate your coffee routine with the Keurig K-Supreme Plus Smart, the ultimate brewing experience. Its large 78 oz reservoir and modern brushed stainless steel accents ensure ample coffee and sleek style. The advanced BrewID system guarantees a perfect cup with every brew. With multistream extraction technology, this single-serve brewer delivers a rich and full-bodied taste. The K-Supreme Plus Smart is perfect for coffee lovers who demand the best – upgrade to a world of flavors with this user-friendly and premium brewing system.</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>3072</v>
+        <v>3939</v>
       </c>
       <c r="G19" t="n">
         <v>197</v>
       </c>
       <c r="H19" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
-        <v>1.048e-05</v>
+        <v>1.042e-05</v>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -1735,21 +1735,21 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Power your healthy lifestyle with the ultimate blending experience! The Vitamix 5200 Blender is a game-changer, with a 2-hp motor that effortlessly blends even the toughest ingredients. Tailor your blend with variable speed control, and enjoy the convenience of self-cleaning. Crafted with sustainably sourced materials and a BPA-free Tritan jar, you can trust this blender to deliver. Plus, a 7-year warranty gives you peace of mind. Elevate your nutrition and your kitchen game with the Vitamix 5200 – a smart investment in your health and happiness.</t>
+          <t>Experience culinary perfection with the Vitamix 5200 Blender, trusted by professionals and home cooks alike. Its powerful 2-hp motor and variable speed control ensure smooth blending, from silky soups to icy treats. The self-cleaning design and BPA-free Tritan jar keep maintenance easy. Plus, with a 7-year warranty, you can invest with confidence. And, rest assured that this high-performance blender is sustainably sourced. Elevate your kitchen with this incredible blend of performance, quality, and sustainability.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3457</v>
+        <v>4119</v>
       </c>
       <c r="G20" t="n">
         <v>197</v>
       </c>
       <c r="H20" t="n">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
-        <v>1.12e-05</v>
+        <v>1.03e-05</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
@@ -1783,11 +1783,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>"Meet the Dyson V15 Detect Vacuum, the cutting-edge cleaning companion for a healthier home. Equipped with a state-of-the-art laser that identifies and captures even the tiniest dust particles, you can trust that every surface is thoroughly cleaned. The HEPA filtration system captures 99.97% of microscopic dust, pollen, and allergens. Plus, with 60 minutes of fuss-free run-time and an energy-efficient design, you'll be amazed at how easy it is to keep your space sparkling. Enjoy peace of mind with our 2-year warranty and a cleaner tomorrow."</t>
+          <t>Elevate your cleaning experience with the Dyson V15 Detect Vacuum! This powerful and energy-efficient machine is equipped with a groundbreaking laser dust detection system, revealing hidden dirt and debris. Featuring True Capture HEPA filtration, it captures 99.97% of microscopic particles as small as 0.3 microns. With a 60-minute run-time and high-quality polycarbonate and aluminum construction, you can trust the V15 Detect to deliver superior performance. Plus, enjoy a 2-year warranty for peace of mind. Take the first step towards a cleaner, healthier home today!</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>4823</v>
+        <v>5824</v>
       </c>
       <c r="G21" t="n">
         <v>197</v>
@@ -1831,21 +1831,21 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>"Introducing the future of cleaning, the iRobot Roomba j7+! This cutting-edge robot vac navigates around objects and furniture with ease, thanks to its advanced PrecisionVision navigation system. Plus, with the self-emptying Clean Base, you'll never have to worry about constantly emptying the dustbin. With simple voice control via Alexa and an award-winning design, this robot vac is not only efficient but also stylish. Say goodbye to messy floors and hello to a cleaner, more convenient home with the iRobot Roomba j7+."</t>
+          <t>Meet the ultimate cleaning companion: the iRobot Roomba j7+! This cutting-edge robot vacuum navigates with unparalleled precision, effortlessly avoiding obstacles and getting into tight spaces to leave your floors spotless. With its self-emptying Clean Base, you'll never need to touch dirt and debris again. Simply schedule and control with Alexa, and enjoy the sleek, award-winning design that complements any home. Upgrade to smarter cleaning and spend more time on what matters – not scrubbing floors!</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4688</v>
+        <v>4523</v>
       </c>
       <c r="G22" t="n">
         <v>192</v>
       </c>
       <c r="H22" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
-        <v>1.056e-05</v>
+        <v>9.780000000000001e-06</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
@@ -1879,21 +1879,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>"Stay inspired and hydrated on-the-go with the Yeti Rambler 20 oz Tumbler. This highly insulated, compact hot and iced beverage container is designed to keep your drinks at the perfect temperature for hours. The leak-proof MagSlider lid and kitchen-grade stainless steel construction ensure durability and easy cleaning. Take it with you on your favorite hike or daily commute - the 5-year warranty gives you confidence in its performance and longevity."</t>
+          <t>Meet the Yeti Rambler 20 oz Tumbler, your new go-to for hot and cold drinks. This double-wall vacuum insulated tumbler keeps liquids at the perfect temperature, while the MagSlider lid provides a comfortable, spill-proof sipping experience. Crafted from durable kitchen-grade stainless steel, this compact tumbler is built to last. And with a 5-year warranty backing it up, you can enjoy your favorite drinks with confidence. Take it on-the-go with the Yeti Rambler, your new trusted companion for hot and cold beverages.</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2696</v>
+        <v>25888</v>
       </c>
       <c r="G23" t="n">
         <v>195</v>
       </c>
       <c r="H23" t="n">
-        <v>91</v>
+        <v>117</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
-        <v>9.36e-06</v>
+        <v>1.092e-05</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
@@ -1927,21 +1927,21 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Stay refreshed on-the-go with the Stanley Quencher H2.0! This 40 oz behemoth keeps your drinks icy for hours due to its vacuum insulated design. The unique flow-state lid and cup-holder friendly design make it a perfect companion for daily hydration. Built to last, it's crafted from recycled stainless steel and backed by a lifetime warranty. With long-lasting battery power to keep the insulation running, you can enjoy your favorite beverages wherever life takes you.</t>
+          <t>Stay hydrated on-the-go with the Stanley Quencher H2.0, a refreshing powerhouse featuring a 40 oz capacity. The vacuum-insulated design keeps drinks hot or cold for hours, while the flow-state lid lets you easily take a sip. Compact and cup-holder friendly, it's perfect for daily adventures. Built to last from recycled stainless steel, this accessory comes with a lifetime warranty, giving you peace of mind as you pour your favorite beverages from one cup-lasting companion.</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3220</v>
+        <v>5433</v>
       </c>
       <c r="G24" t="n">
         <v>195</v>
       </c>
       <c r="H24" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>9.6e-06</v>
+        <v>9.780000000000001e-06</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
@@ -1975,21 +1975,21 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Elevate your hydration game with the Hydro Flask 32 oz Wide Mouth! This premium water bottle features TempShield insulation, keeping drinks hot or cold for hours. Its pro-grade stainless steel construction is durable and resistant to rust, while the Color Last powder coat ensures vibrant colors won't fade. Compact and easy to stash, this bottle makes a perfect daily companion. Plus, with a lifetime warranty, you can trust it'll keep up with your adventurous lifestyle for years to come. Stay refreshed and sustainable!</t>
+          <t>"Stay hydrated and energized on-the-go with the Hydro Flask 32 oz Wide Mouth! Made from pro-grade stainless steel, this insulated powerhouse keeps drinks at the perfect temperature for hours. Our TempShield technology ensures your coffee stays hot and your iced tea stays cold. And with a lifetime warranty, you can trust this bottle will be by your side for all your adventures. Available in a range of colors, this compact design fits neatly into any bag or backpack."</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>5404</v>
+        <v>3773</v>
       </c>
       <c r="G25" t="n">
         <v>189</v>
       </c>
       <c r="H25" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
-        <v>9.9e-06</v>
+        <v>9.480000000000001e-06</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -2023,21 +2023,21 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>"Elevate your hydration game with the Contigo Autoseal West Loop 16 oz! This compact beauty boasts a spill-proof lid and double-wall insulation, keeping your drinks hot or cold for hours. Crafted from durable stainless steel, it's the perfect companion for on-the-go adventures. Plus, a lifetime warranty gives you peace of mind. Ditch the hassle and upgrade to a hassle-free hydration experience with the Contigo Autoseal West Loop - your new favorite travel mug!"</t>
+          <t>Take your daily commute or outdoor adventures to the next level with the Contigo Autoseal West Loop 16 oz. This compact, stainless steel water bottle features a leak-proof autoseal lid and double-wall insulation to keep drinks hot or cold for hours. Trust in the lifetime warranty and enjoy the freedom to take your water on-the-go. Perfectly sized for your car cup holder or desk, this bottle is a must-have for anyone looking to stay hydrated in style.</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>6905</v>
+        <v>4095</v>
       </c>
       <c r="G26" t="n">
         <v>192</v>
       </c>
       <c r="H26" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="n">
-        <v>9.780000000000001e-06</v>
+        <v>9.6e-06</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
@@ -2071,21 +2071,21 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>"Take your runs to the next level with the Nike Air Zoom Pegasus 40! Delivering a smooth ride with React foam and Zoom Air units, these shoes will keep you energized mile after mile. The breathable engineered mesh upper ensures comfort and flexibility, while the gearshift into energy efficiency means you can tackle long distances without fatigue. Built to last with a 2-year manufacturer warranty, the Pegasus 40 is the ultimate choice for performance-driven runners."</t>
+          <t>Get ready to take your run to the next level with the Nike Air Zoom Pegasus 40! This high-performance shoe is engineered with a lightweight React foam midsole for exceptional cushioning and energy return, while Zoom Air units provide a responsive bounce. The engineered mesh upper keeps you cool and dry with a breathable fit. Energy-efficient and built to last, this shoe comes with a 2-year manufacturer warranty. Upgrade your game with the Pegasus 40 - shop now and experience the thrill of a faster, more efficient you!</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>5844</v>
+        <v>4247</v>
       </c>
       <c r="G27" t="n">
         <v>192</v>
       </c>
       <c r="H27" t="n">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="n">
-        <v>9.480000000000001e-06</v>
+        <v>1.026e-05</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -2119,21 +2119,21 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>"Take your running performance to new heights with the Adidas Ultraboost Light! This sleek shoe features a Light BOOST midsole for maximum energy return, a Primeknit+ upper for a secure and comfortable fit, and Continental rubber for superior traction. With a 4.7/5 rating from satisfied customers, you can trust this shoe to deliver results. Plus, a 2-year manufacturer warranty gives you peace of mind. Upgrade your runs and elevate your style with the Adidas Ultraboost Light - order yours today!"</t>
+          <t>Elevate your running game with the Adidas Ultraboost Light! This high-performance shoe features a Light BOOST midsole for superb energy return, making every step feel like springtime. The Primeknit+ upper provides a snug, customizable fit that encourages freedom of movement. With Continental rubber outsoles, you'll enjoy stable traction on any surface. Plus, with a 4.7-star rating and 2-year warranty, you can trust the quality and support. Upgrade your runs with the Adidas Ultraboost Light - your feet will thank you!</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>5797</v>
+        <v>4435</v>
       </c>
       <c r="G28" t="n">
         <v>199</v>
       </c>
       <c r="H28" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
-        <v>1.034e-05</v>
+        <v>1.07e-05</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -2167,21 +2167,21 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Stay warm and light on any adventure with The North Face ThermoBall Eco Jacket. This compact wonder features efficient ThermoBall insulation, shedding snow and rain with ease, thanks to its DWR finish. Made from 100% recycled nylon, it's a responsible choice for the planet. Plus, with a lifetime warranty, you can trust this jacket to be your reliable companion through snowstorms, hikes, and all your outdoor escapades. Wear it with confidence and enjoy the freedom.</t>
+          <t>Stay warm and stay green with The North Face ThermoBall Eco Jacket! This innovative eco-jacket combines synthetic ThermoBall insulation with a durable DWR finish, keeping you cozy in any weather. Plus, it's ultra-compact and lightweight for easy packing. Made from 100% recycled nylon, you can feel good about your purchase. And, with a lifetime warranty, you can trust that this jacket will be your reliable companion for years to come. Perfect for outdoor enthusiasts and eco-conscious consumers alike.</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>6086</v>
+        <v>3854</v>
       </c>
       <c r="G29" t="n">
         <v>192</v>
       </c>
       <c r="H29" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="n">
-        <v>9.72e-06</v>
+        <v>1.002e-05</v>
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
@@ -2215,21 +2215,21 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>"Explore the world with confidence and style in the Patagonia Black Hole 32 L Backpack. Durable and weather-resistant, this bag withstands the elements while keeping your gear dry. A laptop sleeve and padded straps ensure comfortable carrying. Made from 100% recycled polyester ripstop, you'll be reducing your eco-footprint while staying on top of your day. Whether hiking, commuting, or traveling, this backpack is designed for adventure. Enjoy a lifetime warranty and peace of mind with Patagonia's quality guarantee."</t>
+          <t>Hit the trails in comfort and confidence with the Patagonia Black Hole 32 L Backpack. Built with 100% recycled polyester ripstop, this rugged bag keeps you dry and their impact on the planet to a minimum. Plus, with a laptop sleeve and padded straps, you'll stay organized and comfortable on even the longest hikes. And if it doesn't meet your expectations, Patagonia's got you covered: this bag's protected by their lifetime warranty. Grab your gear and get going!</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3697</v>
+        <v>5604</v>
       </c>
       <c r="G30" t="n">
         <v>194</v>
       </c>
       <c r="H30" t="n">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="n">
-        <v>1.024e-05</v>
+        <v>9.94e-06</v>
       </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
@@ -2263,21 +2263,21 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>"Meet the ultimate travel companion - the Osprey Farpoint 40! This incredibly efficient pack is designed for long-haul adventures, with a stowaway harness and laptop sleeve to keep you organized and on the move. Made from durable 450D recycled nylon, it's also kind to the planet. Plus, it meets carry-on size requirements for seamless travel. Experience the freedom to roam with confidence - and do it sustainably - thanks to Osprey's lifetime warranty. Discover the Farpoint 40 today!"</t>
+          <t>"The Osprey Farpoint 40 is a versatile and reliable travel companion, perfect for your next adventure. Its stowaway harness and laptop sleeve ensure comfortable and organized transport, while its carry-on size makes it ideal for gate-to-gate travel. Crafted from 450D recycled nylon, this eco-friendly pack is also energy-efficient. Plus, Osprey's lifetime warranty gives you peace of mind. Whether you're exploring foreign lands or traversing the country, the Farpoint 40 is the perfect bag to carry your essentials in style."</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>4821</v>
+        <v>11268</v>
       </c>
       <c r="G31" t="n">
         <v>192</v>
       </c>
       <c r="H31" t="n">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="n">
-        <v>1.026e-05</v>
+        <v>1.056e-05</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -2311,21 +2311,21 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>"Get ready for the ultimate LEGO Star Wars experience! The 75192 Millennium Falcon is a breathtaking build that's sure to delight even the most seasoned fan. With 7,541 pieces and a detailed interior, you'll be immersed in the iconic spaceship's intricacies. Plus, enjoy long-lasting play with the included minifigs. Built to last with high-quality ABS plastic bricks, this set comes with a lifetime guarantee. Join the Rebel Alliance and create an unforgettable LEGO adventure!"</t>
+          <t>"Embark on an epic adventure with the ultimate LEGO Star Wars souvenir - the Millennium Falcon 75192! With an astonishing 7541 pieces, this colossal model promises to captivate Star Wars enthusiasts of all ages. Discover the intricate details and spacious interior, complete with 5 minifigures. Built to endure with long-lasting battery life, this iconic aircraft will outlast your love for the Force. Lifetime replacement of missing bricks guarantees peace of mind. May the brick be with you!"</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>5076</v>
+        <v>5062</v>
       </c>
       <c r="G32" t="n">
         <v>198</v>
       </c>
       <c r="H32" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="n">
-        <v>9.840000000000001e-06</v>
+        <v>9.96e-06</v>
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -2359,21 +2359,21 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bring a touch of serenity to your space with the LEGO Icons Botanical Orchid 10311. This intricately designed floral set features 608 pieces and allows you to adjust the blooms for a unique look. Made from high-quality ABS plastic bricks, it's durable and long-lasting. Choose from multiple color options to match your home decor. Plus, with a lifetime warranty, you can enjoy your beautiful orchid with peace of mind. Create a stunning centerpiece or gift it to a nature lover – the possibilities are endless!</t>
+          <t>"Bloom with beauty and creativity! Our LEGO Icons Botanical Orchid 10311 is a stunning decorative set that brings the tropical charm of this iconic flower to your home. With 608 pieces and adjustable blooms, you can customize the look to suit your style. Made from high-quality ABS plastic bricks, this set is sure to delight plant enthusiasts and LEGO fans alike. Plus, with our lifetime warranty, you can enjoy this lovely orchid for years to come."</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>4464</v>
+        <v>4497</v>
       </c>
       <c r="G33" t="n">
         <v>195</v>
       </c>
       <c r="H33" t="n">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="n">
-        <v>1.026e-05</v>
+        <v>9.54e-06</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -2407,21 +2407,21 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Elevate your reading experience with the Kindle Paperwhite 11th Gen. This compact e-reader boasts a 6.8" glare-free display, perfect for devouring your favorite books in any light. Enjoy up to 10 weeks of battery life, thanks to its power-efficient design and USB-C charging. Our commitment to sustainability is reflected in the e-reader's recycled plastic design. With a 1-year limited warranty, you can focus on what matters most - getting lost in a great story.</t>
+          <t>Immerse yourself in a world of reading with the Kindle Paperwhite 11th Gen. This sleek device boasts a 6.8" glare-free display, perfect for reading anywhere, anytime. Enjoy up to 10 weeks of battery life and access your library with a single charge via USB-C. Made from recycled plastic, you can feel good about your purchase. All backed by a 1-year limited warranty for peace of mind. Whether you're a bookworm or a casual reader, this is the ultimate travel companion. Start exploring new stories today!</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3079</v>
+        <v>3964</v>
       </c>
       <c r="G34" t="n">
         <v>198</v>
       </c>
       <c r="H34" t="n">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="n">
-        <v>1.008e-05</v>
+        <v>1.074e-05</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -2455,21 +2455,21 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Meet the Kobo Libra 2, the ultimate reading companion! With its stunning 7" E Ink Carta display, you'll enjoy a crisp, glare-free reading experience on any device. Take your audiobooks on the go with seamless Bluetooth connectivity. Plus, this lightweight e-reader's waterproof design means you can read in peace, puddle-free. Weighing in at a mere [insert weight], it's the perfect travel buddy. Enjoy peace of mind with a 1-year limited warranty – happy reading!</t>
+          <t>Meet the Kobo Libra 2, the ultimate reading companion! This sleek e-reader boasts a crisp 7" E Ink Carta display, perfect for long reading sessions. With Bluetooth connectivity, you can enjoy audiobooks without needing to charge the device (since it's waterproof, rain or shine!). Plus, its light weight ensures hours of comfortable reading on the go. With a 1-year limited warranty, you can read without worry. Upgrade your reading experience today and get lost in your favorite stories!</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3265</v>
+        <v>2966</v>
       </c>
       <c r="G35" t="n">
         <v>198</v>
       </c>
       <c r="H35" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="n">
-        <v>1.038e-05</v>
+        <v>1.02e-05</v>
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
@@ -2503,21 +2503,21 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Elevate your outdoor adventures with the Anker Soundcore Motion+ Speaker! Enjoy powerful 30W audio and crystal-clear Hi-Res sound wherever you go. Made from a durable aluminum grille and designed to withstand the elements with IPX7 waterproofing, this portable speaker can keep the music flowing in the rain or shine. Plus, its energy efficiency ensures long-lasting playtime. Backed by an 18-month warranty, you can trust that your Soundcore Motion+ will keep delivering big sound with minimal fuss.</t>
+          <t>"Get ready to elevate your outdoor experiences with the Anker Soundcore Motion+ Speaker! This robust wireless speaker pumps out 30W of Hi-Res audio, ensuring you feel the beat wherever you go. Built with an aluminum grille and IPX7 waterproof rating, it can withstand the elements and harsh conditions. Plus, its energy-efficient design means you can enjoy great sound without sacrificing battery life. With an 18-month warranty, you can trust the quality of this remarkable speaker."</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3349</v>
+        <v>3568</v>
       </c>
       <c r="G36" t="n">
         <v>193</v>
       </c>
       <c r="H36" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="n">
-        <v>1.016e-05</v>
+        <v>9.74e-06</v>
       </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -2551,21 +2551,21 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Take your music on the go without limits with the Sonos Move 2! This rugged speaker boasts a stunning 24-hour battery life, keeping the rhythm playing all day and all night. Thanks to automatic Trueplay, your tunes are optimized for wherever you are - indoors, outdoors, or on the move. With seamless WiFi and Bluetooth connectivity, streaming is effortless. Plus, its shock-resistant shell keeps it safe from bumps and drops. Enjoy unbeatable sound with peace of mind - 4.7/5 stars don't lie!</t>
+          <t>Take your music anywhere with the Sonos Move 2! This portable powerhouse packs amazing sound into a shock-resistant shell, delivering rich, clear audio both indoors and out. With up to 24 hours of battery life, you can enjoy your favorite beats all day long. And with automatic Trueplay tuning, you can trust that your sound is always perfect. With its seamless WiFi and Bluetooth connectivity, stream from your favorite services with ease. Your audio adventures just got a whole lot more enjoyable!</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>5285</v>
+        <v>4743</v>
       </c>
       <c r="G37" t="n">
         <v>199</v>
       </c>
       <c r="H37" t="n">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="n">
-        <v>1.046e-05</v>
+        <v>9.92e-06</v>
       </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2599,21 +2599,21 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Elevate your home with the Philips Hue White &amp; Color Ambiance Starter Kit! This limited edition kit lets you choose from 16 million colors and experience seamless voice control with Bluetooth and Zigbee technology. Imagine setting the perfect ambiance with just the sound of your voice. "Goodnight" gives way to a soothing blue hue, while "Party Time" explodes into a vibrant display. With its durable plastic bulbs and 2-year warranty, confidence comes included. Get ready to unleash a world of color and convenience!</t>
+          <t>Unlock a world of color and convenience with the Philips Hue White &amp; Color Ambiance Starter Kit! This limited edition starter kit features 16 million colors, can be controlled via Bluetooth &amp; Zigbee, and is even voice-friendly. Easily transform your space with a palette of endless possibilities. Plus, with a 2-year limited warranty, you can trust your new Hue lights to bring ambiance to your home for years to come. Experience the ultimate in smart lighting - order yours today!</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>3281</v>
+        <v>3517</v>
       </c>
       <c r="G38" t="n">
         <v>195</v>
       </c>
       <c r="H38" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="n">
-        <v>1.014e-05</v>
+        <v>9.660000000000001e-06</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
@@ -2647,21 +2647,21 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Experience lightning-fast, seamless WiFi across your entire home with the TP-Link Deco XE75 Mesh WiFi 6E. This tri-band AXE5400 system covers up to 7,200 sq ft with just 3 units, ensuring strong connections everywhere. Plus, with long-lasting battery life, these nodes can stay online for months at a time without needing a recharge. Backed by a 2-year warranty, you can trust your WiFi to stay strong and stable with Deco XE75.</t>
+          <t>Elevate your home network with the TP-Link Deco XE75 Mesh WiFi 6E. This powerful tri-band system covers up to 7,200 square feet with a single 3-pack setup, ensuring seamless coverage and lag-free browsing. The battery-powered design provides long-lasting reliability, while the durable plastic build withstands the rigors of daily life. Backed by a 2-year limited warranty, this mesh system gives you peace of mind, providing you with a robust and future-proof WiFi solution for all your connected devices.</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>3160</v>
+        <v>21889</v>
       </c>
       <c r="G39" t="n">
         <v>205</v>
       </c>
       <c r="H39" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="n">
-        <v>1.034e-05</v>
+        <v>1.076e-05</v>
       </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
@@ -2695,21 +2695,21 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Elevate your home's security with the Eufy Video Doorbell Dual. Equipped with a dual camera, this device provides a wider view of your entrance, detecting packages and keeping an eye on your belongings. With 2K resolution, you'll enjoy crisp and clear footage day or night. Powered by a long-lasting battery, this doorbell is convenient and hassle-free. Enjoy peace of mind with a 1-year limited warranty, knowing you're protected against defects and malfunctions. Upgrade your home's security today!</t>
+          <t>Elevate your home's security with the Eufy Video Doorbell Dual! This innovative device features two cameras, giving you a comprehensive view of your surroundings. Plus, with 2K resolution, you'll capture every detail. Package detection and motion tracking keep you informed of any unusual activity. And with a long-lasting battery, you'll enjoy peace of mind without the hassle of recharging. Backed by a 1-year limited warranty, you can trust that you're protected. Stay safe and secure with the Eufy Video Doorbell Dual.</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>4308</v>
+        <v>3240</v>
       </c>
       <c r="G40" t="n">
         <v>193</v>
       </c>
       <c r="H40" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="n">
-        <v>1.028e-05</v>
+        <v>1.064e-05</v>
       </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
@@ -2743,21 +2743,21 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Elevate your home security with the limited edition Blink Outdoor 4. This compact, weather-resistant camera boasts stunning 1080p HD footage, giving you crystal-clear insight into your surroundings. With a 2-year battery life, you can enjoy peace of mind without worrying about frequent recharging. And with our 1-year limited warranty, you can trust that your investment is protected. Upgrade your home security and experience sleek, reliable protection with the Blink Outdoor 4.</t>
+          <t>"Experience the freedom of wireless outdoor security with the limited edition Blink Outdoor 4. Capture crisp 1080p HD footage, day or night, and enjoy up to 2 years of battery life on a single charge. Durable and weather-resistant, this plug-and-play camera is perfect for any outdoor space. Backed by a 1-year limited warranty, you can trust the Blink Outdoor 4 to provide seamless video recording and peace of mind, keeping you connected to what matters most."</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3356</v>
+        <v>2350</v>
       </c>
       <c r="G41" t="n">
         <v>190</v>
       </c>
       <c r="H41" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="n">
-        <v>9.56e-06</v>
+        <v>9.800000000000001e-06</v>
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
@@ -2791,21 +2791,21 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Elevate your gaming experience with the Corsair K100 RGB Keyboard! This premium keyboard boasts rapid responsiveness thanks to Cherry MX Speed switches and 4000 Hz polling, giving you an unparalleled advantage. The durable aluminum frame stands up to intense gaming sessions, while its large capacity layout provides ample space for your fingers. Plus, a 2-year warranty gives you peace of mind. Get ready to dominate the competition with unmatched speed and performance.</t>
+          <t>Take your gaming and typing experience to the next level with the Corsair K100 RGB Keyboard! Equipped with Cherry MX Speed switches for lightning-fast actuation, you'll enjoy lightning-quick response times. The aluminum frame is both durable and stylish, while 4000 Hz polling ensures seamless connectivity. Backed by a 2-year warranty, you can play with precision and confidence. Upgrade your setup with the K100 and feel the difference for yourself – immersive gaming, elevated.</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>2143</v>
+        <v>2180</v>
       </c>
       <c r="G42" t="n">
         <v>192</v>
       </c>
       <c r="H42" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="n">
-        <v>9.18e-06</v>
+        <v>9.659999999999999e-06</v>
       </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
@@ -2839,21 +2839,21 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Elevate your productivity with the Logitech MX Master 3S. This high-performance mouse boasts a 8K DPI sensor for accurate tracking and smooth navigation. The MagSpeed scroll enables lightning-fast transitioning between scrolling and superb precision. Connect wirelessly via either Bolt or Bluetooth for seamless productivity. Choose from a range of stylish options to suit your workspace. With a 1-year limited warranty, you can trust your new mouse to deliver. Experience the difference it makes in your work and daily life.</t>
+          <t>Elevate your productivity with the Logitech MX Master 3S, a precision wireless mouse engineered for peak performance. Its 8K DPI sensor tracks every movement with uncanny accuracy, while the MagSpeed scroll wheel lets you zip through long documents or web pages with ease. Easily switch between devices with Bolt, Logitech's proprietary wireless technology, or pair via Bluetooth. Available in a range of stylish colors, this mouse is a must-have for creators, professionals, and anyone who demands the best.</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2630</v>
+        <v>2403</v>
       </c>
       <c r="G43" t="n">
         <v>195</v>
       </c>
       <c r="H43" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="n">
-        <v>9.96e-06</v>
+        <v>1.002e-05</v>
       </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
@@ -2887,21 +2887,21 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Take your gaming to the next level with the Razer DeathAdder V3 Pro! This sleek and precise mouse is designed to give you the speed and accuracy you need to dominate the competition. Weighing in at just 63g, it's an ultralight champion that glides effortlessly across any surface. With a long-lasting battery and 30K DPI Focus Pro sensor, you'll enjoy lightning-fast tracking and hours of uninterrupted play. Plus, our 2-year warranty gives you peace of mind. Upgrade your game today!</t>
+          <t>Elevate your gaming experience with the Razer DeathAdder V3 Pro. Weighing in at just 63g, this ultralight mouse glides effortlessly across your surface, providing precision and control. Powered by the 30K DPI Focus Pro sensor, you'll enjoy lightning-fast movements and pinpoint accuracy. Plus, enjoy long-lasting battery life without the need for frequent recharging. Backed by a 2-year warranty, you can focus on dominating the competition, not replacing your gear. Upgrade your gaming arsenal today and experience the ultimate in mouse performance.</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3040</v>
+        <v>2357</v>
       </c>
       <c r="G44" t="n">
         <v>196</v>
       </c>
       <c r="H44" t="n">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="n">
-        <v>1.046e-05</v>
+        <v>1.088e-05</v>
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
@@ -2935,21 +2935,21 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>"Unleash the power of your system with the Samsung 980 Pro 2 TB NVMe SSD! This lightning-fast storage drive is powered by PCIe 4.0 technology, delivering breathtaking read speeds of up to 7,000 MB/s. With its durable nickel coating and long-lasting battery, you can rely on it for your most demanding tasks. Built with high-quality PCB and NAND flash components, this SSD is backed by a 5-year limited warranty. Say goodbye to wait times and hello to seamless performance!"</t>
+          <t>Amplify your computer's performance with the Samsung 980 Pro 2 TB NVMe SSD! This powerhouse drive leverages PCIe 4.0 to reach blistering speeds of up to 7,000 MB/s read, ensuring seamless app launching and smooth gaming. With a nickel coating for added durability and a long-lasting battery, you can tackle demanding tasks and storage-intensive projects with confidence. Backed by a 5-year warranty, this SSD is built to last - upgrade your system and unlock new possibilities!</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>3756</v>
+        <v>2270</v>
       </c>
       <c r="G45" t="n">
         <v>206</v>
       </c>
       <c r="H45" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="n">
-        <v>1.048e-05</v>
+        <v>1.036e-05</v>
       </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
@@ -2983,21 +2983,21 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>"Store your entire digital life in one place with the Seagate Portable 5 TB HDD. Easily transport and expand your storage space with this compact and plug-and-play drive. With USB 3.0 speeds, you'll get fast data transfer rates. The 2.5" form factor fits neatly in your pocket or bag, making it perfect for on-the-go use. Enjoy confident storage with a 1-year limited warranty. Say goodbye to storage worries and get the peace of mind that comes with this reliable 4.7/5-rated external hard drive."</t>
+          <t>Take your digital life on the go! Our Seagate Portable 5 TB HDD stores up to 2,500 hours of your favorite movies or 1,200,000 songs. With a simple plug-and-play design and USB 3.0 speed, transferring files is effortless. Perfect for photographers, videographers, or anyone with extensive digital collections. Durable and compact, this 2.5″ portable drive fits easily in a bag. Rest assured with a 4.7-star rating and 1-year limited warranty. Get organized, get free – bring your portable HDD today!</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3353</v>
+        <v>2390</v>
       </c>
       <c r="G46" t="n">
         <v>204</v>
       </c>
       <c r="H46" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="n">
-        <v>1.098e-05</v>
+        <v>1.128e-05</v>
       </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
@@ -3031,21 +3031,21 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Capture life's big moments with confidence. The SanDisk Extreme PRO 128 GB SDXC card is designed to keep up with you. With read speeds of up to 200 MB/s, you can quickly transfer and free up space on your device. Water-resistant and built to withstand the toughest conditions, this long-lasting card is perfect for photographers, videographers, and adventure-seekers alike. Backed by a lifetime limited warranty, you can trust it to perform whenever duty calls.</t>
+          <t>Capture life's most epic moments with the SanDisk Extreme PRO 128 GB SDXC card. Shoot non-stop with UHS-I U3 speeds of 200 MB/s read, and rely on its waterproof design for peace of mind. With a long-lasting battery life, you'll never miss a shot. Store thousands of photos and 4K videos with ample storage. Backed by a lifetime limited warranty, this card is designed to keep up with your adventurous lifestyle, allowing you to focus on what matters most - the moment.</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>2462</v>
+        <v>1992</v>
       </c>
       <c r="G47" t="n">
         <v>195</v>
       </c>
       <c r="H47" t="n">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="n">
-        <v>9.780000000000001e-06</v>
+        <v>1.032e-05</v>
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
@@ -3079,21 +3079,21 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Invest in high-performance computing with the Kingston Fury Beast 32 GB DDR5. This cutting-edge memory features a blazing 6000 MT/s speed and Intel XMP 3.0 for effortless overclocking. Our low-profile heat spreader keeps cool, even under intense loads, while its energy-efficient design minimizes power consumption. Backed by a lifetime warranty, this reliable solution is perfect for demanding gamers, enthusiasts, and professionals who crave seamless performance and peace of mind. Upto 64 gigs total capacity.</t>
+          <t>Give your rig a boost with the Kingston Fury Beast 32 GB DDR5! This beast of a memory module runs at a scorching 6000 MT/s, making it perfect for gamers and content creators who demand the best. With Intel XMP 3.0, you can easily tweak your settings for optimal performance. Our low-profile heat spreader keeps things cool, while aluminum construction ensures durability. Plus, with a lifetime warranty, we've got your back - upgrade to the Fury Beast today!</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>2794</v>
+        <v>1765</v>
       </c>
       <c r="G48" t="n">
         <v>200</v>
       </c>
       <c r="H48" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="n">
-        <v>1.024e-05</v>
+        <v>1.018e-05</v>
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
@@ -3127,21 +3127,21 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>"Elevate your gaming and content experience with the Acer Predator XB273U 27" Monitor. This massive display boasts a 2560x1440 resolution, rapid 170Hz refresh rate, and HDR400 color technology, delivering crisp details and immersive visuals. With G-Sync Compatible for smooth performance and a sturdy metal and plastic frame, you'll be fully engaged. Plus, enjoy 3 years of worry-free use with our included warranty. Upgrade to exceptional visuals and a seamless gaming experience today!"</t>
+          <t>Take your gaming to the next level with the Acer Predator XB273U 27" Monitor! This beastly display boasts a 170Hz IPS panel with 2560*1440 resolution for crystal-clear visuals. Plus, with HDR400 and G-Sync Compatible, you'll be immersed in smooth, vibrant action. The large screen and robust metal stand ensure a commanding presence on your desk. Enjoy peace of mind with Acer's 3-year warranty. Upgrade your gaming setup today and experience the thrill of unparalleled performance!</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>3222</v>
+        <v>2633</v>
       </c>
       <c r="G49" t="n">
         <v>203</v>
       </c>
       <c r="H49" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="n">
-        <v>1.018e-05</v>
+        <v>1.036e-05</v>
       </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -3175,21 +3175,21 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>"Unleash your creativity with the BenQ PD2725U 27" monitor. Featuring 4K UHD IPS technology, this stunning display delivers vibrant colors and razor-sharp images. With 98% P3 color gamut, you'll enjoy a stunning range of hues and saturation. The powerful Thunderbolt 3 port enables lightning-fast transfer speeds, while the sleek metal stand adds a touch of sophistication. Plus, a 3-year warranty gives you peace of mind. Upgrade your workspace with this incredible monitor and experience the difference for yourself."</t>
+          <t>"Bring your creative vision to life with the BenQ PD2725U 27" Monitor! This stunning display boasts an impressive 4K UHD IPS panel with 98% P3 color gamut, ensuring vibrant and accurate colors. With Thunderbolt 3 connectivity, you can transmit data at lightning-fast speeds. Durable and stylish, the metal stand holds fast to the sleek design. Plus, you're protected with a 3-year warranty. Upgrade your workflow with this versatile monitor, perfect for videographers, graphic designers, and anyone who demands exceptional visuals."</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>4550</v>
+        <v>3153</v>
       </c>
       <c r="G50" t="n">
         <v>202</v>
       </c>
       <c r="H50" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="n">
-        <v>1.082e-05</v>
+        <v>1.1e-05</v>
       </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
@@ -3223,21 +3223,21 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Unleash your creativity with the ASUS ProArt PA278QV Monitor! This stunning 27" IPS display features a precise 2560*1440 resolution and 100% sRGB color coverage, ensuring that your designs and colors are faithfully reproduced. The Calman Verified certification guarantees accuracy, while its lightweight metal stand makes it effortless to set up. Backed by a 3-year warranty, this impressive monitor is designed to inspire confidence and precision. Take your artwork to the next level with the ASUS ProArt PA278QV.</t>
+          <t>Elevate your creative workflow with the ASUS ProArt PA278QV Monitor! This 27" stunning display boasts a crystal-clear 2560*1440 IPS panel, delivering 100% sRGB color accuracy for breathtaking visuals. Engineered for professionals, it meets rigorous Calman Verified standards. The sleek metal stand is both sturdy and lightweight, ensuring ergonomic comfort. Plus, with a 3-year warranty, you can focus on bringing your vision to life, worry-free. Unlock your full creative potential with the ProArt PA278QV – precision, power, and unparalleled viewing experience await.</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>5688</v>
+        <v>2734</v>
       </c>
       <c r="G51" t="n">
         <v>202</v>
       </c>
       <c r="H51" t="n">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="n">
-        <v>1.064e-05</v>
+        <v>1.136e-05</v>
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>

</xml_diff>